<commit_message>
Update versioned master parameter workbook
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -57420,4 +57420,296 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a32518fee107c04aa9bd7948c0d3f18">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e97db55af52189d57b3fce0d0bdbaea8" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
+    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD8B92E4-A62E-4C3D-ABB7-B1C8056BB11B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6EEC841-3638-4C83-A17D-B41FFD8905C4}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37AD3F2D-24B3-4F2A-92A9-16CAFF700971}"/>
 </file>
</xml_diff>

<commit_message>
Harden RPI orchestration and machine setup IO
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -46457,7 +46457,7 @@
       <c r="S608" s="4" t="n"/>
       <c r="T608" s="4" t="n"/>
     </row>
-    <row r="609" ht="180" customHeight="1">
+    <row r="609" ht="270" customHeight="1">
       <c r="A609" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46524,11 +46524,11 @@
       <c r="P609" s="24" t="n"/>
       <c r="Q609" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Etiketten- bzw. Traegerbandbreite in 1/10 mm. Der Wert definiert zugleich die Sollposition der beiden Etikettenanschlaege: der rechte Nullpunkt liegt von oben gesehen an der rechten Bandkante, daher entspricht 20.0 mm dem Sollwert 200 und 55.0 mm dem Sollwert 550 fuer Einlauf- und Auslaufanschlag. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Der Wert definiert auch wo die beiden Etiekttenanschläge positioniert werden. Stelle Dir vor dass die Etikette von oben gesehen im Produktionsbetrieb von unten nach oben läuft und dass der 0-Punkt der Bahn auf der das Etikettenträgerband läuft ganz rechts ist. Wenn eine 20mm breite Etikette hier im format angegeben wird, müssen die beiden anschläge auf 200 (20mm) fahren, bei einer 55mm Etikette auf 550 usw.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="610" ht="150" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Etiketten- bzw. Traegerbandbreite in 1/10 mm. Der Wert definiert zugleich die Sollposition der beiden Etikettenanschlaege: der rechte Nullpunkt liegt von oben gesehen an der rechten Bandkante, daher entspricht 20.0 mm dem Sollwert 200 und 55.0 mm dem Sollwert 550 fuer Einlauf- und Auslaufanschlag. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="610" ht="225" customHeight="1">
       <c r="A610" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46595,11 +46595,11 @@
       <c r="P610" s="38" t="n"/>
       <c r="Q610" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Soll-Etikettenlaenge ohne Gap in 1/10 mm. Der ESP muss die real gemessene Etikettenlaenge mit MAP0040 vergleichen; bei zu kurzer Laenge wird MAE0025 gesetzt, bei zu langer Laenge MAE0026. Der Raspi behandelt diese beiden Fehler als Produktionspause statt als Purge/Not-Stop. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Etikettenlänge wird für die Erfassungs/Sensorüberwachung der Etiekttenlänge verwendet. Der Parameter hängt zusammen mit MAP0040. Weicht die gemessene Länge im System mehr als MAP0040 nach oben/unten ab, wird ein entsprechender Fehler ausgelöst und die Produktion pausiert.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="611" ht="210" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Soll-Etikettenlaenge ohne Gap in 1/10 mm. Der ESP muss die real gemessene Etikettenlaenge mit MAP0040 vergleichen; bei zu kurzer Laenge wird MAE0025 gesetzt, bei zu langer Laenge MAE0026. Der Raspi behandelt diese beiden Fehler als Produktionspause statt als Purge/Not-Stop. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="611" ht="285" customHeight="1">
       <c r="A611" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46666,11 +46666,11 @@
       <c r="P611" s="24" t="n"/>
       <c r="Q611" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Druckposition in X-/Querrichtung auf dem Etikett. Fuer die Portalachse X gilt eine Umkehrlogik: ein positiver Druckpositionswert verschiebt den Tisch in negative X-Richtung, ein negativer Wert in positive X-Richtung. Die zusaetzliche Korrektur MAP0005 wird vorher auf den Druckpositionswert addiert. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Dies ist die Druckposition auf der Etikette in Querrichtung (wieder von oben gesehen rechts)ist der 0-Punkt. Das hat in der Steuerung folgende Funktion: Je nachdem welcher drucker (Laser/TTO) aktiv ist (bestimmt durch MAP0016) wird der tisch in X-Richtung weiter nach vorne bewegt. 0 heisst dabei dass die X-Achse im Produktionsbetrieb auf 0 geht und ein wert vom parameter hier von 20 bedeutet dass die X-Achse auf -20 (-2mmgeht ) und bei einem Wert von -20 muss die X-achse um 20 (2mm) nach vorne hier herrscht also ein Umkehrwert.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="612" ht="240" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Druckposition in X-/Querrichtung auf dem Etikett. Fuer die Portalachse X gilt eine Umkehrlogik: ein positiver Druckpositionswert verschiebt den Tisch in negative X-Richtung, ein negativer Wert in positive X-Richtung. Die zusaetzliche Korrektur MAP0005 wird vorher auf den Druckpositionswert addiert. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="612" ht="285" customHeight="1">
       <c r="A612" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46737,11 +46737,11 @@
       <c r="P612" s="38" t="n"/>
       <c r="Q612" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Druckposition in Y-/Laufrichtung auf dem Etikett. Der konkrete Stopppunkt ergibt sich aus MAP0018 fuer Laser oder MAP0019 fuer TTO plus MAP0004 und plus Korrektur MAP0006. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Dies ist die Druckposition auf der Etikette in Längsrichtung (wieder von oben gesehen oben)ist der 0-Punkt. Das hat in der Steuerung folgende Funktion: Die Distanz MAP0018 bzw. MAP0019 (je nach aktivem Drucker) beschreibt die Position der Etikette in laufrichtung ganz am anfang (von oben gesehen). Der Wert 0 bedeutet somit, dass das Etiekttenband zum drucken bei genau Erfassungsanfang+MAP0018 oder MAP0019 + 0 stoppen muss. Steht hier z.b.50, soll der druck von oben gesehen in laufrichtung 5mm nach unten versetzt werden, was bedeutet, dass der stop-punkt zum drucken nun bei Erfassungsanfang des jewiligen Etiketts+MAP0018 oder MAP0019 + 50 stoppen muss.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="613" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Druckposition in Y-/Laufrichtung auf dem Etikett. Der konkrete Stopppunkt ergibt sich aus MAP0018 fuer Laser oder MAP0019 fuer TTO plus MAP0004 und plus Korrektur MAP0006. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="613" ht="150" customHeight="1">
       <c r="A613" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46808,11 +46808,11 @@
       <c r="P613" s="24" t="n"/>
       <c r="Q613" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als zusaetzliche Korrektur auf die X-Druckposition. Er wird auf MAP0003 addiert, bevor daraus die invertierte X-Achskorrektur fuer den Tisch gebildet wird. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Hier kann eine zusätliche Korrektur auf den X-Wert vorgenommen werden (dieser wird auf den X-Wert aufaddiert).. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP darf ihn im Prozess aktiv verwenden und - falls fachlich vorgesehen - auch setzen oder rueckmelden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="614" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als zusaetzliche Korrektur auf die X-Druckposition. Er wird auf MAP0003 addiert, bevor daraus die invertierte X-Achskorrektur fuer den Tisch gebildet wird. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP darf ihn im Prozess aktiv verwenden und - falls fachlich vorgesehen - auch setzen oder rueckmelden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="614" ht="150" customHeight="1">
       <c r="A614" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46879,11 +46879,11 @@
       <c r="P614" s="38" t="n"/>
       <c r="Q614" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als zusaetzliche Korrektur auf die Y-Druckposition. Er wird auf MAP0004 addiert und beeinflusst damit den exakten Druck-Stoppweg in Laufrichtung. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Hier kann eine zusätliche Korrektur auf den Y-Wert vorgenommen werden (dieser wird auf den Y-Wert aufaddiert).. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP darf ihn im Prozess aktiv verwenden und - falls fachlich vorgesehen - auch setzen oder rueckmelden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="615" ht="150" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als zusaetzliche Korrektur auf die Y-Druckposition. Er wird auf MAP0004 addiert und beeinflusst damit den exakten Druck-Stoppweg in Laufrichtung. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP darf ihn im Prozess aktiv verwenden und - falls fachlich vorgesehen - auch setzen oder rueckmelden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="615" ht="195" customHeight="1">
       <c r="A615" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -46950,11 +46950,11 @@
       <c r="P615" s="24" t="n"/>
       <c r="Q615" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Materialdicke bzw. Produktions-Z-Position des Tisches in 1/10 mm. Zusammen mit der Nullpunktkorrektur MAP0028 ergibt er den Z-Sollwert fuer den Produktionsbetrieb. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Dieser wert Steuert die Z-Achse vom Tisch im Produktionsbetrieb und beschreibt die Etiekttendicke. Ein Wert von 1 bedeutet die Z-Achse muss im Produktionsbetrieb auf 1 fahren, ein wert von 50 bedeutet die Z-Achse muss im Produktionsbetrieb auf 50 fahren,. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="616" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Materialdicke bzw. Produktions-Z-Position des Tisches in 1/10 mm. Zusammen mit der Nullpunktkorrektur MAP0028 ergibt er den Z-Sollwert fuer den Produktionsbetrieb. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="616" ht="180" customHeight="1">
       <c r="A616" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47021,11 +47021,11 @@
       <c r="P616" s="38" t="n"/>
       <c r="Q616" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Querposition des Etikettenerfassungs-Sensors im Produktionsbetrieb in mm. Fuer die Motor-/Achslogik wird er in 1/10 mm umgerechnet und mit der Nullpunktkorrektur MAP0029 kombiniert. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Das ist die Position der Verstellachse für den Etiekttenerfassungssensor im Produktionsbetrieb in mm.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="617" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Querposition des Etikettenerfassungs-Sensors im Produktionsbetrieb in mm. Fuer die Motor-/Achslogik wird er in 1/10 mm umgerechnet und mit der Nullpunktkorrektur MAP0029 kombiniert. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="617" ht="165" customHeight="1">
       <c r="A617" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47092,11 +47092,11 @@
       <c r="P617" s="24" t="n"/>
       <c r="Q617" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Querposition des Entnahme-/Kontrollsensors im Produktionsbetrieb in mm. Fuer die Motor-/Achslogik wird er in 1/10 mm umgerechnet und mit der Nullpunktkorrektur MAP0030 kombiniert. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Das ist die Position der Verstellachse für den ENtnahme/Kontrollensor im Produktionsbetrieb in mm.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="618" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Querposition des Entnahme-/Kontrollsensors im Produktionsbetrieb in mm. Fuer die Motor-/Achslogik wird er in 1/10 mm umgerechnet und mit der Nullpunktkorrektur MAP0030 kombiniert. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="618" ht="180" customHeight="1">
       <c r="A618" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47163,11 +47163,11 @@
       <c r="P618" s="38" t="n"/>
       <c r="Q618" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als X-/Quer-Leseposition der Material-Kontrollkamera. Er beschreibt die formatabhaengige Kameraposition; die mechanische Achskorrektur fuer diese Kamera wird separat ueber MAP0033 bzw. die Motor-Sollposition MAP0060 beruecksichtigt. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Das ist die Position der Verstellachse für den Etiekttenerfassungssensor im Produktionsbetrieb in mm.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="619" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als X-/Quer-Leseposition der Material-Kontrollkamera. Er beschreibt die formatabhaengige Kameraposition; die mechanische Achskorrektur fuer diese Kamera wird separat ueber MAP0033 bzw. die Motor-Sollposition MAP0060 beruecksichtigt. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="619" ht="165" customHeight="1">
       <c r="A619" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47234,11 +47234,11 @@
       <c r="P619" s="24" t="n"/>
       <c r="Q619" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Y-/Laengs-Leseposition der Material-Kontrollkamera. Der Wert ist ein Prozessbezug fuer Trigger-/Auswertefenster und nicht die Motor-ID-5-Querachse selbst. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Das ist die Position der Verstellachse für die Materialkontrollkamera im Produktionsbetrieb in mm.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="620" ht="120" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Y-/Laengs-Leseposition der Material-Kontrollkamera. Der Wert ist ein Prozessbezug fuer Trigger-/Auswertefenster und nicht die Motor-ID-5-Querachse selbst. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="620" ht="165" customHeight="1">
       <c r="A620" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47305,11 +47305,11 @@
       <c r="P620" s="38" t="n"/>
       <c r="Q620" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Y-/Laengs-Leseposition der OCR-/Verifizierungs-Kamera. Die Kamera ist aktuell nicht als eigene Verstellachse modelliert; der Wert bleibt aber fuer Prozessfenster und spaetere Verifikation relevant. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Das ist die Position der Verstellachse für OCE Verifikationskamera im Produktionsbetrieb in mm.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="621" ht="210" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Y-/Laengs-Leseposition der OCR-/Verifizierungs-Kamera. Die Kamera ist aktuell nicht als eigene Verstellachse modelliert; der Wert bleibt aber fuer Prozessfenster und spaetere Verifikation relevant. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="621" ht="315" customHeight="1">
       <c r="A621" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47376,11 +47376,11 @@
       <c r="P621" s="24" t="n"/>
       <c r="Q621" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Rollenkern-Typ fuer Auf- und Abwicklung (0=76 mm, 1=100 mm). Die vorhandene Hardware kann den Kern nicht sicher direkt erkennen; eine Plausibilisierung ueber Wicklerbewegung und Rollenfuellstand ist theoretisch denkbar, aber noch nicht freigegeben. Deshalb wird der Wert vorerst nur als lesbarer Format-/Materialhinweis an den ESP gespiegelt und nicht aktiv fuer Regelentscheidungen verwendet. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Das ist der Parameter für den Typ des aufgespannten Etiekttenrollenkerns auf der Auf-und ABwicklung. Momentan wird das noch nicht verwendet und es ist auch nicht sicher ob der Parameter drin bleibt., da nicht sicher ist, ob anhand der Bewegungen des auf-und abwicklers kontrolliert werden kann, welcher Kern (76 oder 100mm) aktuell aufgespannt ist. Aufgabe: Finde heraus ob das technisch machbar ist mit der vorhandenen Hardware und schreibe hier das Ergebnis rein, verändere noch nichts am Code diesbezüglich.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: OFF/ON. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
-        </is>
-      </c>
-    </row>
-    <row r="622" ht="225" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Rollenkern-Typ fuer Auf- und Abwicklung (0=76 mm, 1=100 mm). Die vorhandene Hardware kann den Kern nicht sicher direkt erkennen; eine Plausibilisierung ueber Wicklerbewegung und Rollenfuellstand ist theoretisch denkbar, aber noch nicht freigegeben. Deshalb wird der Wert vorerst nur als lesbarer Format-/Materialhinweis an den ESP gespiegelt und nicht aktiv fuer Regelentscheidungen verwendet. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: OFF/ON. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="622" ht="255" customHeight="1">
       <c r="A622" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -47447,7 +47447,7 @@
       <c r="P622" s="38" t="n"/>
       <c r="Q622" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Soll-Transportgeschwindigkeit des Etikettenbands. Im kontinuierlichen Lasermodus ist er die Druck-/Bandgeschwindigkeit; in allen getakteten Modi ist er die Vorzugsgeschwindigkeit zwischen den Druckpositionen. Der ESP nutzt ihn fuer Taktbewegungen und dynamische Nachregelung, der Raspi fuer Transparenz, Logging und Bedienung. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Der Parameter ist hier noch nicht vollständig korrekt beschrieben. IM Kontinuierlichen Lasermodus (nicht getakteter Betrieb) ist dies die Vorzugsgeschwindigkeit der Eteikette über den Etiekttenantrieb. In jedem anderen Modus ist dieser Parameter die Vorzugsgeschwindigkeit zwischen den Druckpositionen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm/s. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+          <t>KI: Ich verstehe diesen Parameter als Soll-Transportgeschwindigkeit des Etikettenbands. Im kontinuierlichen Lasermodus ist er die Druck-/Bandgeschwindigkeit; in allen getakteten Modi ist er die Vorzugsgeschwindigkeit zwischen den Druckpositionen. Der ESP nutzt ihn fuer Taktbewegungen und dynamische Nachregelung, der Raspi fuer Transparenz, Logging und Bedienung. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: mm/s. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
         </is>
       </c>
     </row>
@@ -48019,7 +48019,7 @@
         </is>
       </c>
     </row>
-    <row r="631" ht="105" customHeight="1">
+    <row r="631" ht="135" customHeight="1">
       <c r="A631" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48078,7 +48078,7 @@
       </c>
       <c r="M631" s="23" t="inlineStr">
         <is>
-          <t>Vorwarnung Etikettenfüllstand bei Abwicklung</t>
+          <t>Vorwarnung Etikettenfuellstand bei Abwicklung (bald leer)</t>
         </is>
       </c>
       <c r="N631" s="23" t="n"/>
@@ -48086,11 +48086,11 @@
       <c r="P631" s="24" t="n"/>
       <c r="Q631" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Vorwarnschwelle fuer den Abwickler in Prozent. Wenn MAS0008 unter diesen Wert faellt, soll daraus die passende Warnung fuer Materialende entstehen. Der ESP liest diesen Wert fuer die Wickler-/Prozesslogik, Microtom liest ihn als eingestellte Schwelle. Microtom soll diesen Wert nur lesen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: %. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="632" ht="105" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Vorwarnschwelle fuer den Abwickler in Prozent Restfuellstand. Wenn MAS0008 kleiner/gleich diesem Wert ist, ist die Abwickelrolle bald leer und die passende Wickler-/Materialwarnung muss aktiv werden. Der ESP liest diesen Wert fuer die Wickler-/Prozesslogik, Microtom liest ihn als eingestellte Schwelle. Microtom soll diesen Wert nur lesen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: %. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="632" ht="150" customHeight="1">
       <c r="A632" s="31" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48103,17 +48103,17 @@
       </c>
       <c r="C632" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>70</t>
         </is>
       </c>
       <c r="D632" s="7" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E632" s="7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>95</t>
         </is>
       </c>
       <c r="F632" s="31" t="inlineStr">
@@ -48149,7 +48149,7 @@
       </c>
       <c r="M632" s="39" t="inlineStr">
         <is>
-          <t>Vorwarnung Etikettenfüllstand bei Aufwicklung</t>
+          <t>Vorwarnung Etikettenfuellstand bei Aufwicklung (bald voll)</t>
         </is>
       </c>
       <c r="N632" s="37" t="n"/>
@@ -48157,7 +48157,7 @@
       <c r="P632" s="38" t="n"/>
       <c r="Q632" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Vorwarnschwelle fuer den Aufwickler in Prozent. Wenn MAS0009 unter diesen Wert faellt, soll daraus die passende Warnung fuer Materialende bzw. Rollenfuellstand entstehen. Der ESP liest diesen Wert fuer die Wickler-/Prozesslogik, Microtom liest ihn als eingestellte Schwelle. Microtom soll diesen Wert nur lesen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: %. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe diesen Parameter als Vorwarnschwelle fuer den Aufwickler in Prozent Rollenfuellstand. Wenn MAS0009 groesser/gleich diesem Wert ist, ist die Aufwickelrolle bald voll und die passende Wickler-/Materialwarnung muss aktiv werden. Default ist 95 %, also Warnung im Bereich 95-100 %. Alte/gespiegelte Werte kleiner/gleich 50 werden in der Wickler-Firmware uebergangsweise als Restreserve bis voll interpretiert, z.B. 5 bedeutet Warnung ab 95 %. Der ESP liest diesen Wert fuer die Wickler-/Prozesslogik, Microtom liest ihn als eingestellte Schwelle. Microtom soll diesen Wert nur lesen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: %. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
     </row>
@@ -48303,7 +48303,7 @@
         </is>
       </c>
     </row>
-    <row r="635" ht="165" customHeight="1">
+    <row r="635" ht="225" customHeight="1">
       <c r="A635" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48370,11 +48370,11 @@
       <c r="P635" s="24" t="n"/>
       <c r="Q635" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Portalachse X. Die programmierte Motor-Nullposition bleibt die Grundstellung; dieser Wert verschiebt den fachlichen Nullpunkt fuer alle X-bezogenen Berechnungen. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="636" ht="165" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Portalachse X. Die programmierte Motor-Nullposition bleibt die Grundstellung; dieser Wert verschiebt den fachlichen Nullpunkt fuer alle X-bezogenen Berechnungen. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="636" ht="225" customHeight="1">
       <c r="A636" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48441,11 +48441,11 @@
       <c r="P636" s="21" t="n"/>
       <c r="Q636" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Portalachse Z. Die programmierte Motor-Nullposition bleibt die Grundstellung; dieser Wert verschiebt den fachlichen Nullpunkt fuer alle Z-bezogenen Berechnungen. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="637" ht="180" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Portalachse Z. Die programmierte Motor-Nullposition bleibt die Grundstellung; dieser Wert verschiebt den fachlichen Nullpunkt fuer alle Z-bezogenen Berechnungen. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="637" ht="225" customHeight="1">
       <c r="A637" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48512,11 +48512,11 @@
       <c r="P637" s="24" t="n"/>
       <c r="Q637" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Querachse fuer den Etikettenerfassungs-Sensor. Alle Sensorpositionen fuer diese Achse werden relativ zu diesem korrigierten Nullpunkt betrachtet. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="638" ht="180" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Querachse fuer den Etikettenerfassungs-Sensor. Alle Sensorpositionen fuer diese Achse werden relativ zu diesem korrigierten Nullpunkt betrachtet. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="638" ht="210" customHeight="1">
       <c r="A638" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48583,11 +48583,11 @@
       <c r="P638" s="21" t="n"/>
       <c r="Q638" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Querachse fuer den Entnahme-/Kontrollsensor. Alle Sensorpositionen fuer diese Achse werden relativ zu diesem korrigierten Nullpunkt betrachtet. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="639" ht="180" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Querachse fuer den Entnahme-/Kontrollsensor. Alle Sensorpositionen fuer diese Achse werden relativ zu diesem korrigierten Nullpunkt betrachtet. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="639" ht="210" customHeight="1">
       <c r="A639" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48654,11 +48654,11 @@
       <c r="P639" s="24" t="n"/>
       <c r="Q639" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur des Etikettenanschlags am Einlauf. Die aus MAP0001 abgeleitete Bandbreitenposition wird um diese Korrektur verschoben. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="640" ht="180" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur des Etikettenanschlags am Einlauf. Die aus MAP0001 abgeleitete Bandbreitenposition wird um diese Korrektur verschoben. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="640" ht="210" customHeight="1">
       <c r="A640" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48725,11 +48725,11 @@
       <c r="P640" s="21" t="n"/>
       <c r="Q640" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur des Etikettenanschlags am Auslauf. Die aus MAP0001 abgeleitete Bandbreitenposition wird um diese Korrektur verschoben. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="641" ht="180" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur des Etikettenanschlags am Auslauf. Die aus MAP0001 abgeleitete Bandbreitenposition wird um diese Korrektur verschoben. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="641" ht="210" customHeight="1">
       <c r="A641" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48796,11 +48796,11 @@
       <c r="P641" s="24" t="n"/>
       <c r="Q641" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Material-Kontrollkamera-Querachse. Die formatabhaengige Kameraposition wird relativ zu diesem korrigierten Nullpunkt betrachtet. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="642" ht="180" customHeight="1">
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur der Material-Kontrollkamera-Querachse. Die formatabhaengige Kameraposition wird relativ zu diesem korrigierten Nullpunkt betrachtet. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="642" ht="210" customHeight="1">
       <c r="A642" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -48867,7 +48867,7 @@
       <c r="P642" s="21" t="n"/>
       <c r="Q642" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur des Laser-Schutzblechs. Die Schutzblechachse bleibt parametrierbar, auch wenn der Laserprozess spaeter finalisiert wird. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Die Grundstellung ist eigentlich immer bei der programmierten 0 - Position des jeweiligen Motors. Dieser Wert versteht sich als korrekturangabe auf den eigentlichen 0-Punkt. Wird hier ein anderer Wert als 0 eingegeben, gild dieser korrigierte wert als 0-Punkt für alle anderen Parameter und Funktionen, welche sich auf diesen 0 Punkt beziehen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe diesen Parameter als Nullpunktkorrektur des Laser-Schutzblechs. Die Schutzblechachse bleibt parametrierbar, auch wenn der Laserprozess spaeter finalisiert wird. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
     </row>
@@ -49155,7 +49155,7 @@
         </is>
       </c>
     </row>
-    <row r="647" ht="165" customHeight="1">
+    <row r="647" ht="240" customHeight="1">
       <c r="A647" s="15" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -49222,7 +49222,7 @@
       <c r="P647" s="24" t="n"/>
       <c r="Q647" s="22" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe diesen Parameter als Freigabe fuer automatische Rueckspulung nach Produktionsstop. Wenn der Wert 1 ist, wird nach Produktionsstop und Rueckspul-Taster bis zum Ursprungspunkt zurueckgespult und erst danach die Produktion abgeschlossen; bei 0 gilt die Produktion ohne Rueckspulung als abgeschlossen. Aus der ergaenzten Fachbeschreibung wurde ausgewertet: Ist dieser Wert 1, wird nach dem Produktionsstop automatisch (nach drücken des Rückspul-Tasters) die Etiektte an den Ursprungspunkt zurückgespult und erst dann wird die Produktion abgeschlossen. Ist der Wert 0, erfolgt keine Rückspulung und die Produktion gilt nach dem Produktionsstop als abgeschlossen.. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: OFF/ON. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
+          <t>KI: Ich verstehe diesen Parameter als Freigabe fuer automatische Rueckspulung nach Produktionsstop. Wenn der Wert 1 ist, wird nach Produktionsstop und Rueckspul-Taster bis zum Ursprungspunkt zurueckgespult und erst danach die Produktion abgeschlossen; bei 0 gilt die Produktion ohne Rueckspulung als abgeschlossen. Microtom soll diesen Wert fuehrend schreiben koennen. Der ESP soll ihn aus der Raspi-/Microtom-Seite lesen bzw. gespiegelt bekommen, aber nicht fuehrend schreiben. Einheit bzw. Wertebereich laut Tabelle: OFF/ON. Der Wert ist formatrelevant und muss beim Formatwechsel konsistent mitgezogen werden.</t>
         </is>
       </c>
     </row>
@@ -49723,7 +49723,7 @@
         </is>
       </c>
     </row>
-    <row r="655" ht="120" customHeight="1">
+    <row r="655" ht="135" customHeight="1">
       <c r="A655" s="8" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -50990,7 +50990,7 @@
       <c r="P673" s="22" t="n"/>
       <c r="Q673" s="22" t="n"/>
     </row>
-    <row r="674" ht="135" customHeight="1">
+    <row r="674" ht="150" customHeight="1">
       <c r="A674" s="10" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -51064,7 +51064,7 @@
         </is>
       </c>
     </row>
-    <row r="675" ht="135" customHeight="1">
+    <row r="675" ht="150" customHeight="1">
       <c r="A675" s="10" t="inlineStr">
         <is>
           <t>MAP</t>
@@ -57007,118 +57007,408 @@
       </c>
     </row>
     <row r="758" hidden="1">
-      <c r="A758" s="10" t="n"/>
-      <c r="B758" s="8" t="n"/>
-      <c r="C758" s="43" t="n"/>
-      <c r="D758" s="11" t="n"/>
-      <c r="E758" s="11" t="n"/>
-      <c r="F758" s="15" t="n"/>
-      <c r="G758" s="15" t="n"/>
-      <c r="H758" s="15" t="n"/>
-      <c r="I758" s="15" t="n"/>
-      <c r="J758" s="15" t="n"/>
-      <c r="K758" s="22" t="n"/>
-      <c r="L758" s="22" t="n"/>
-      <c r="M758" s="22" t="n"/>
-      <c r="N758" s="22" t="n"/>
-      <c r="O758" s="22" t="n"/>
-      <c r="P758" s="22" t="n"/>
-      <c r="Q758" s="22" t="n"/>
+      <c r="A758" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B758" s="8" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="C758" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D758" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E758" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F758" s="29" t="n"/>
+      <c r="G758" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="H758" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I758" s="29" t="inlineStr">
+        <is>
+          <t>uint8</t>
+        </is>
+      </c>
+      <c r="J758" s="29" t="inlineStr">
+        <is>
+          <t>Temporaerer IBN/Test Prozessbefehl</t>
+        </is>
+      </c>
+      <c r="K758" s="28" t="n"/>
+      <c r="L758" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M758" s="28" t="inlineStr">
+        <is>
+          <t>0=Stop, 1=Wickler einmessen+Messfahrt, 2=Taktbetrieb, 3=Vorziehen kontinuierlich, 4=Zurueckspulen kontinuierlich</t>
+        </is>
+      </c>
+      <c r="N758" s="28" t="n"/>
+      <c r="O758" s="28" t="n"/>
+      <c r="P758" s="28" t="n"/>
+      <c r="Q758" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0001 als temporaeren IBN-/Testbefehl von Microtom an den Raspi. Der Raspi uebersetzt diesen Wert in produktionsnahe Startkommandos fuer ESP32-PLC und Wickler. Dieser Parameter ist ausdruecklich nur fuer Inbetriebnahme/Test vorgesehen und muss spaeter entfernt oder durch produktive MAS/MAP-Ablaufbefehle ersetzt werden. Der ESP soll ihn gemaess Masterliste nicht direkt als normalen Parameter verwenden. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="R758" s="4" t="n"/>
+      <c r="S758" s="4" t="n"/>
+      <c r="T758" s="4" t="n"/>
     </row>
     <row r="759" hidden="1">
-      <c r="A759" s="10" t="n"/>
-      <c r="B759" s="8" t="n"/>
-      <c r="C759" s="43" t="n"/>
-      <c r="D759" s="11" t="n"/>
-      <c r="E759" s="11" t="n"/>
-      <c r="F759" s="15" t="n"/>
-      <c r="G759" s="15" t="n"/>
-      <c r="H759" s="15" t="n"/>
-      <c r="I759" s="15" t="n"/>
-      <c r="J759" s="15" t="n"/>
-      <c r="K759" s="22" t="n"/>
-      <c r="L759" s="22" t="n"/>
-      <c r="M759" s="22" t="n"/>
-      <c r="N759" s="22" t="n"/>
-      <c r="O759" s="22" t="n"/>
-      <c r="P759" s="22" t="n"/>
-      <c r="Q759" s="22" t="n"/>
+      <c r="A759" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B759" s="8" t="inlineStr">
+        <is>
+          <t>0002</t>
+        </is>
+      </c>
+      <c r="C759" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D759" s="12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E759" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F759" s="29" t="inlineStr">
+        <is>
+          <t>1/10mm</t>
+        </is>
+      </c>
+      <c r="G759" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="H759" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I759" s="29" t="inlineStr">
+        <is>
+          <t>uint16</t>
+        </is>
+      </c>
+      <c r="J759" s="29" t="inlineStr">
+        <is>
+          <t>Temporaere Takt-/Labellaenge</t>
+        </is>
+      </c>
+      <c r="K759" s="28" t="n"/>
+      <c r="L759" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M759" s="28" t="inlineStr">
+        <is>
+          <t>Labelweg fuer getakteten Testbetrieb in 1/10 mm</t>
+        </is>
+      </c>
+      <c r="N759" s="28" t="n"/>
+      <c r="O759" s="28" t="n"/>
+      <c r="P759" s="28" t="n"/>
+      <c r="Q759" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0002 als temporaere Labellaenge bzw. Taktstrecke fuer den IBN-Test. Default 1000 bedeutet 100.0 mm. Spaeter kommt dieser Wert aus Rezept-/Formatdaten und Etiketteneinmessung, nicht mehr aus einem MAC-Testparameter. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="R759" s="4" t="n"/>
+      <c r="S759" s="4" t="n"/>
+      <c r="T759" s="4" t="n"/>
     </row>
     <row r="760" hidden="1">
-      <c r="A760" s="10" t="n"/>
-      <c r="B760" s="8" t="n"/>
-      <c r="C760" s="43" t="n"/>
-      <c r="D760" s="11" t="n"/>
-      <c r="E760" s="11" t="n"/>
-      <c r="F760" s="15" t="n"/>
-      <c r="G760" s="15" t="n"/>
-      <c r="H760" s="15" t="n"/>
-      <c r="I760" s="15" t="n"/>
-      <c r="J760" s="15" t="n"/>
-      <c r="K760" s="22" t="n"/>
-      <c r="L760" s="22" t="n"/>
-      <c r="M760" s="22" t="n"/>
-      <c r="N760" s="22" t="n"/>
-      <c r="O760" s="22" t="n"/>
-      <c r="P760" s="22" t="n"/>
-      <c r="Q760" s="22" t="n"/>
+      <c r="A760" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B760" s="8" t="inlineStr">
+        <is>
+          <t>0003</t>
+        </is>
+      </c>
+      <c r="C760" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D760" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="E760" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="F760" s="29" t="inlineStr">
+        <is>
+          <t>mm/s</t>
+        </is>
+      </c>
+      <c r="G760" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="H760" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I760" s="29" t="inlineStr">
+        <is>
+          <t>uint16</t>
+        </is>
+      </c>
+      <c r="J760" s="29" t="inlineStr">
+        <is>
+          <t>Temporaere Vorzugsgeschwindigkeit</t>
+        </is>
+      </c>
+      <c r="K760" s="28" t="n"/>
+      <c r="L760" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M760" s="28" t="inlineStr">
+        <is>
+          <t>Sollgeschwindigkeit fuer kontinuierlichen und getakteten IBN-Testbetrieb</t>
+        </is>
+      </c>
+      <c r="N760" s="28" t="n"/>
+      <c r="O760" s="28" t="n"/>
+      <c r="P760" s="28" t="n"/>
+      <c r="Q760" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0003 als temporaere Vorzugsgeschwindigkeit fuer Motor 3 im IBN-Test. Wird kein neuer Wert gesetzt, verwendet der Raspi den zuletzt gespeicherten Wert. Produktiv wird die Geschwindigkeit ueber MAP0014 bzw. die Betriebsart vorgegeben. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="R760" s="4" t="n"/>
+      <c r="S760" s="4" t="n"/>
+      <c r="T760" s="4" t="n"/>
     </row>
     <row r="761" hidden="1">
-      <c r="A761" s="10" t="n"/>
-      <c r="B761" s="8" t="n"/>
-      <c r="C761" s="43" t="n"/>
-      <c r="D761" s="11" t="n"/>
-      <c r="E761" s="11" t="n"/>
-      <c r="F761" s="15" t="n"/>
-      <c r="G761" s="15" t="n"/>
-      <c r="H761" s="15" t="n"/>
-      <c r="I761" s="15" t="n"/>
-      <c r="J761" s="15" t="n"/>
-      <c r="K761" s="22" t="n"/>
-      <c r="L761" s="22" t="n"/>
-      <c r="M761" s="22" t="n"/>
-      <c r="N761" s="22" t="n"/>
-      <c r="O761" s="22" t="n"/>
-      <c r="P761" s="22" t="n"/>
-      <c r="Q761" s="22" t="n"/>
+      <c r="A761" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B761" s="8" t="inlineStr">
+        <is>
+          <t>0004</t>
+        </is>
+      </c>
+      <c r="C761" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D761" s="12" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E761" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F761" s="29" t="inlineStr">
+        <is>
+          <t>mm/s2</t>
+        </is>
+      </c>
+      <c r="G761" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="H761" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I761" s="29" t="inlineStr">
+        <is>
+          <t>uint16</t>
+        </is>
+      </c>
+      <c r="J761" s="29" t="inlineStr">
+        <is>
+          <t>Temporaere Transport-Rampe</t>
+        </is>
+      </c>
+      <c r="K761" s="28" t="n"/>
+      <c r="L761" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M761" s="28" t="inlineStr">
+        <is>
+          <t>Beschleunigung/Verzoegerung fuer Motor 3 im IBN-Testbetrieb</t>
+        </is>
+      </c>
+      <c r="N761" s="28" t="n"/>
+      <c r="O761" s="28" t="n"/>
+      <c r="P761" s="28" t="n"/>
+      <c r="Q761" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0004 als temporaere Rampe fuer Beschleunigung und Bremsung des Etikettenantriebs im IBN-Test. Produktiv wird diese Vorgabe aus Maschinen- bzw. Formatparametern abgeleitet und darf den Etikettenschlupf nicht erhoehen. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s2. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="R761" s="4" t="n"/>
+      <c r="S761" s="4" t="n"/>
+      <c r="T761" s="4" t="n"/>
     </row>
     <row r="762" hidden="1">
-      <c r="A762" s="10" t="n"/>
-      <c r="B762" s="8" t="n"/>
-      <c r="C762" s="43" t="n"/>
-      <c r="D762" s="11" t="n"/>
-      <c r="E762" s="11" t="n"/>
-      <c r="F762" s="15" t="n"/>
-      <c r="G762" s="15" t="n"/>
-      <c r="H762" s="15" t="n"/>
-      <c r="I762" s="15" t="n"/>
-      <c r="J762" s="15" t="n"/>
-      <c r="K762" s="22" t="n"/>
-      <c r="L762" s="22" t="n"/>
-      <c r="M762" s="22" t="n"/>
-      <c r="N762" s="22" t="n"/>
-      <c r="O762" s="22" t="n"/>
-      <c r="P762" s="22" t="n"/>
-      <c r="Q762" s="22" t="n"/>
+      <c r="A762" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B762" s="8" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="C762" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D762" s="12" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E762" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F762" s="29" t="inlineStr">
+        <is>
+          <t>1/10mm</t>
+        </is>
+      </c>
+      <c r="G762" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="H762" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I762" s="29" t="inlineStr">
+        <is>
+          <t>uint32</t>
+        </is>
+      </c>
+      <c r="J762" s="29" t="inlineStr">
+        <is>
+          <t>Temporaere kontinuierliche Weglaenge</t>
+        </is>
+      </c>
+      <c r="K762" s="28" t="n"/>
+      <c r="L762" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M762" s="28" t="inlineStr">
+        <is>
+          <t>Weg fuer kontinuierliches Vorziehen/Rueckspulen; 0=endlos bis Stop</t>
+        </is>
+      </c>
+      <c r="N762" s="28" t="n"/>
+      <c r="O762" s="28" t="n"/>
+      <c r="P762" s="28" t="n"/>
+      <c r="Q762" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0005 als temporaere Wegvorgabe fuer kontinuierliches Vorziehen oder Rueckspulen. Default 0 bedeutet endlos fahren bis MAC0001=0. Produktiv wird diese Laenge aus Ablaufzustand, Rueckspulweg oder Bedienhandlung bestimmt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="R762" s="4" t="n"/>
+      <c r="S762" s="4" t="n"/>
+      <c r="T762" s="4" t="n"/>
     </row>
     <row r="763" hidden="1">
-      <c r="A763" s="10" t="n"/>
-      <c r="B763" s="8" t="n"/>
-      <c r="C763" s="43" t="n"/>
-      <c r="D763" s="11" t="n"/>
-      <c r="E763" s="11" t="n"/>
-      <c r="F763" s="15" t="n"/>
-      <c r="G763" s="15" t="n"/>
-      <c r="H763" s="15" t="n"/>
-      <c r="I763" s="15" t="n"/>
-      <c r="J763" s="15" t="n"/>
-      <c r="K763" s="22" t="n"/>
-      <c r="L763" s="22" t="n"/>
-      <c r="M763" s="22" t="n"/>
-      <c r="N763" s="22" t="n"/>
-      <c r="O763" s="22" t="n"/>
-      <c r="P763" s="22" t="n"/>
-      <c r="Q763" s="22" t="n"/>
+      <c r="A763" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B763" s="8" t="inlineStr">
+        <is>
+          <t>0006</t>
+        </is>
+      </c>
+      <c r="C763" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D763" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E763" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F763" s="29" t="inlineStr">
+        <is>
+          <t>Zyklen</t>
+        </is>
+      </c>
+      <c r="G763" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="H763" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I763" s="29" t="inlineStr">
+        <is>
+          <t>uint16</t>
+        </is>
+      </c>
+      <c r="J763" s="29" t="inlineStr">
+        <is>
+          <t>Temporaere Taktzyklus-Anzahl</t>
+        </is>
+      </c>
+      <c r="K763" s="28" t="n"/>
+      <c r="L763" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="M763" s="28" t="inlineStr">
+        <is>
+          <t>Anzahl Takte im Testbetrieb; 0=endlos bis Stop</t>
+        </is>
+      </c>
+      <c r="N763" s="28" t="n"/>
+      <c r="O763" s="28" t="n"/>
+      <c r="P763" s="28" t="n"/>
+      <c r="Q763" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0006 als temporaere Zyklusanzahl fuer den getakteten IBN-Test. Default 20 entspricht einem kurzen Stabilitaetstest; 0 bedeutet laufender Taktbetrieb bis MAC0001=0. Spaeter wird diese Logik durch den echten Produktionsablauf und das Schieberegister ersetzt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: Zyklen. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="R763" s="4" t="n"/>
+      <c r="S763" s="4" t="n"/>
+      <c r="T763" s="4" t="n"/>
     </row>
     <row r="764" hidden="1">
       <c r="A764" s="10" t="n"/>
@@ -57703,13 +57993,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD8B92E4-A62E-4C3D-ABB7-B1C8056BB11B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AD463D1-E757-4D31-B8E8-0F1FA0DA293A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6EEC841-3638-4C83-A17D-B41FFD8905C4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A67F1944-362D-43F5-BE44-588BA96467B0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37AD3F2D-24B3-4F2A-92A9-16CAFF700971}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A096BF9-12F5-4E2F-802A-25F1F6BC033C}"/>
 </file>
</xml_diff>

<commit_message>
Sync parameter defaults from production motors
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
@@ -269,6 +269,7 @@
   </cellStyles>
   <dxfs count="20">
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
@@ -296,7 +297,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
@@ -474,9 +474,8 @@
   <autoFilter ref="A1:R778">
     <filterColumn colId="0" hiddenButton="0" showButton="1">
       <filters>
+        <filter val="MAE"/>
         <filter val="MAP"/>
-        <filter val="MAS"/>
-        <filter val="TTP"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -490,18 +489,18 @@
     <tableColumn id="2" name="Max.:" dataDxfId="14"/>
     <tableColumn id="10" name="Default Value:" dataDxfId="13"/>
     <tableColumn id="4" name="Einheit:" dataDxfId="12"/>
-    <tableColumn id="8" name="Microtom User Range:" dataDxfId="0"/>
-    <tableColumn id="5" name="R/W:" dataDxfId="11"/>
-    <tableColumn id="6" name="ESP32 R/W:" dataDxfId="10"/>
-    <tableColumn id="14" name="Data Type:" dataDxfId="9"/>
-    <tableColumn id="15" name="Name:" dataDxfId="8"/>
-    <tableColumn id="7" name="ZBC Mapping:" dataDxfId="7"/>
-    <tableColumn id="11" name="Format relevant?:" dataDxfId="6"/>
-    <tableColumn id="12" name="Message:" dataDxfId="5"/>
-    <tableColumn id="13" name="Possible Cause:" dataDxfId="4"/>
-    <tableColumn id="17" name="Effects:" dataDxfId="3"/>
-    <tableColumn id="18" name="Remedy:" dataDxfId="2"/>
-    <tableColumn id="19" name="KI-Anweisungen:" dataDxfId="1"/>
+    <tableColumn id="8" name="Microtom User Range:" dataDxfId="11"/>
+    <tableColumn id="5" name="R/W:" dataDxfId="10"/>
+    <tableColumn id="6" name="ESP32 R/W:" dataDxfId="9"/>
+    <tableColumn id="14" name="Data Type:" dataDxfId="8"/>
+    <tableColumn id="15" name="Name:" dataDxfId="7"/>
+    <tableColumn id="7" name="ZBC Mapping:" dataDxfId="6"/>
+    <tableColumn id="11" name="Format relevant?:" dataDxfId="5"/>
+    <tableColumn id="12" name="Message:" dataDxfId="4"/>
+    <tableColumn id="13" name="Possible Cause:" dataDxfId="3"/>
+    <tableColumn id="17" name="Effects:" dataDxfId="2"/>
+    <tableColumn id="18" name="Remedy:" dataDxfId="1"/>
+    <tableColumn id="19" name="KI-Anweisungen:" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -41439,7 +41438,7 @@
         </is>
       </c>
     </row>
-    <row r="528" ht="60" customHeight="1">
+    <row r="528" hidden="1" ht="60" customHeight="1">
       <c r="A528" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41509,7 +41508,7 @@
         </is>
       </c>
     </row>
-    <row r="529" ht="60" customHeight="1">
+    <row r="529" hidden="1" ht="60" customHeight="1">
       <c r="A529" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41581,7 +41580,7 @@
         </is>
       </c>
     </row>
-    <row r="530" ht="60" customHeight="1">
+    <row r="530" hidden="1" ht="60" customHeight="1">
       <c r="A530" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41653,7 +41652,7 @@
         </is>
       </c>
     </row>
-    <row r="531" ht="75" customHeight="1">
+    <row r="531" hidden="1" ht="75" customHeight="1">
       <c r="A531" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41727,7 +41726,7 @@
         </is>
       </c>
     </row>
-    <row r="532" ht="60" customHeight="1">
+    <row r="532" hidden="1" ht="60" customHeight="1">
       <c r="A532" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41799,7 +41798,7 @@
         </is>
       </c>
     </row>
-    <row r="533" ht="45" customHeight="1">
+    <row r="533" hidden="1" ht="45" customHeight="1">
       <c r="A533" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41869,7 +41868,7 @@
         </is>
       </c>
     </row>
-    <row r="534" ht="60" customHeight="1">
+    <row r="534" hidden="1" ht="60" customHeight="1">
       <c r="A534" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -41939,7 +41938,7 @@
         </is>
       </c>
     </row>
-    <row r="535" ht="60" customHeight="1">
+    <row r="535" hidden="1" ht="60" customHeight="1">
       <c r="A535" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42009,7 +42008,7 @@
         </is>
       </c>
     </row>
-    <row r="536" ht="60" customHeight="1">
+    <row r="536" hidden="1" ht="60" customHeight="1">
       <c r="A536" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42079,7 +42078,7 @@
         </is>
       </c>
     </row>
-    <row r="537" ht="75" customHeight="1">
+    <row r="537" hidden="1" ht="75" customHeight="1">
       <c r="A537" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42147,7 +42146,7 @@
         </is>
       </c>
     </row>
-    <row r="538" ht="60" customHeight="1">
+    <row r="538" hidden="1" ht="60" customHeight="1">
       <c r="A538" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42217,7 +42216,7 @@
         </is>
       </c>
     </row>
-    <row r="539" ht="60" customHeight="1">
+    <row r="539" hidden="1" ht="60" customHeight="1">
       <c r="A539" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42289,7 +42288,7 @@
         </is>
       </c>
     </row>
-    <row r="540" ht="60" customHeight="1">
+    <row r="540" hidden="1" ht="60" customHeight="1">
       <c r="A540" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42359,7 +42358,7 @@
         </is>
       </c>
     </row>
-    <row r="541" ht="60" customHeight="1">
+    <row r="541" hidden="1" ht="60" customHeight="1">
       <c r="A541" s="15" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42431,7 +42430,7 @@
         </is>
       </c>
     </row>
-    <row r="542" ht="60" customHeight="1">
+    <row r="542" hidden="1" ht="60" customHeight="1">
       <c r="A542" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42503,7 +42502,7 @@
         </is>
       </c>
     </row>
-    <row r="543" ht="75" customHeight="1">
+    <row r="543" hidden="1" ht="75" customHeight="1">
       <c r="A543" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42575,7 +42574,7 @@
         </is>
       </c>
     </row>
-    <row r="544" ht="60" customHeight="1">
+    <row r="544" hidden="1" ht="60" customHeight="1">
       <c r="A544" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42647,7 +42646,7 @@
         </is>
       </c>
     </row>
-    <row r="545" ht="60" customHeight="1">
+    <row r="545" hidden="1" ht="60" customHeight="1">
       <c r="A545" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42723,7 +42722,7 @@
         </is>
       </c>
     </row>
-    <row r="546" ht="60" customHeight="1">
+    <row r="546" hidden="1" ht="60" customHeight="1">
       <c r="A546" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42799,7 +42798,7 @@
         </is>
       </c>
     </row>
-    <row r="547" ht="60" customHeight="1">
+    <row r="547" hidden="1" ht="60" customHeight="1">
       <c r="A547" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42871,7 +42870,7 @@
         </is>
       </c>
     </row>
-    <row r="548" ht="60" customHeight="1">
+    <row r="548" hidden="1" ht="60" customHeight="1">
       <c r="A548" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -42947,7 +42946,7 @@
         </is>
       </c>
     </row>
-    <row r="549" ht="60" customHeight="1">
+    <row r="549" hidden="1" ht="60" customHeight="1">
       <c r="A549" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43017,7 +43016,7 @@
         </is>
       </c>
     </row>
-    <row r="550" ht="60" customHeight="1">
+    <row r="550" hidden="1" ht="60" customHeight="1">
       <c r="A550" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43090,7 +43089,7 @@
         </is>
       </c>
     </row>
-    <row r="551" ht="60" customHeight="1">
+    <row r="551" hidden="1" ht="60" customHeight="1">
       <c r="A551" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43158,7 +43157,7 @@
         </is>
       </c>
     </row>
-    <row r="552" ht="60" customHeight="1">
+    <row r="552" hidden="1" ht="60" customHeight="1">
       <c r="A552" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43230,7 +43229,7 @@
         </is>
       </c>
     </row>
-    <row r="553" ht="75" customHeight="1">
+    <row r="553" hidden="1" ht="75" customHeight="1">
       <c r="A553" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43300,7 +43299,7 @@
         </is>
       </c>
     </row>
-    <row r="554" ht="60" customHeight="1">
+    <row r="554" hidden="1" ht="60" customHeight="1">
       <c r="A554" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43372,7 +43371,7 @@
         </is>
       </c>
     </row>
-    <row r="555" ht="60" customHeight="1">
+    <row r="555" hidden="1" ht="60" customHeight="1">
       <c r="A555" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43444,7 +43443,7 @@
         </is>
       </c>
     </row>
-    <row r="556" ht="60" customHeight="1">
+    <row r="556" hidden="1" ht="60" customHeight="1">
       <c r="A556" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43514,7 +43513,7 @@
         </is>
       </c>
     </row>
-    <row r="557" ht="60" customHeight="1">
+    <row r="557" hidden="1" ht="60" customHeight="1">
       <c r="A557" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43586,7 +43585,7 @@
         </is>
       </c>
     </row>
-    <row r="558" ht="60" customHeight="1">
+    <row r="558" hidden="1" ht="60" customHeight="1">
       <c r="A558" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43658,7 +43657,7 @@
         </is>
       </c>
     </row>
-    <row r="559" ht="60" customHeight="1">
+    <row r="559" hidden="1" ht="60" customHeight="1">
       <c r="A559" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43730,7 +43729,7 @@
         </is>
       </c>
     </row>
-    <row r="560" ht="60" customHeight="1">
+    <row r="560" hidden="1" ht="60" customHeight="1">
       <c r="A560" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43803,7 +43802,7 @@
         </is>
       </c>
     </row>
-    <row r="561" ht="45" customHeight="1">
+    <row r="561" hidden="1" ht="45" customHeight="1">
       <c r="A561" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43875,7 +43874,7 @@
         </is>
       </c>
     </row>
-    <row r="562" ht="60" customHeight="1">
+    <row r="562" hidden="1" ht="60" customHeight="1">
       <c r="A562" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -43943,7 +43942,7 @@
         </is>
       </c>
     </row>
-    <row r="563" ht="45" customHeight="1">
+    <row r="563" hidden="1" ht="45" customHeight="1">
       <c r="A563" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44013,7 +44012,7 @@
         </is>
       </c>
     </row>
-    <row r="564" ht="45" customHeight="1">
+    <row r="564" hidden="1" ht="45" customHeight="1">
       <c r="A564" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44083,7 +44082,7 @@
         </is>
       </c>
     </row>
-    <row r="565" ht="45" customHeight="1">
+    <row r="565" hidden="1" ht="45" customHeight="1">
       <c r="A565" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44153,7 +44152,7 @@
         </is>
       </c>
     </row>
-    <row r="566" ht="60" customHeight="1">
+    <row r="566" hidden="1" ht="60" customHeight="1">
       <c r="A566" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44223,7 +44222,7 @@
         </is>
       </c>
     </row>
-    <row r="567" ht="60" customHeight="1">
+    <row r="567" hidden="1" ht="60" customHeight="1">
       <c r="A567" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44293,7 +44292,7 @@
         </is>
       </c>
     </row>
-    <row r="568" ht="60" customHeight="1">
+    <row r="568" hidden="1" ht="60" customHeight="1">
       <c r="A568" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44365,7 +44364,7 @@
         </is>
       </c>
     </row>
-    <row r="569" ht="45" customHeight="1">
+    <row r="569" hidden="1" ht="45" customHeight="1">
       <c r="A569" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44437,7 +44436,7 @@
         </is>
       </c>
     </row>
-    <row r="570" ht="45" customHeight="1">
+    <row r="570" hidden="1" ht="45" customHeight="1">
       <c r="A570" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44507,7 +44506,7 @@
         </is>
       </c>
     </row>
-    <row r="571" ht="45" customHeight="1">
+    <row r="571" hidden="1" ht="45" customHeight="1">
       <c r="A571" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44577,7 +44576,7 @@
         </is>
       </c>
     </row>
-    <row r="572" ht="45" customHeight="1">
+    <row r="572" hidden="1" ht="45" customHeight="1">
       <c r="A572" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44649,7 +44648,7 @@
         </is>
       </c>
     </row>
-    <row r="573" ht="60" customHeight="1">
+    <row r="573" hidden="1" ht="60" customHeight="1">
       <c r="A573" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44721,7 +44720,7 @@
         </is>
       </c>
     </row>
-    <row r="574" ht="45" customHeight="1">
+    <row r="574" hidden="1" ht="45" customHeight="1">
       <c r="A574" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44791,7 +44790,7 @@
         </is>
       </c>
     </row>
-    <row r="575" ht="60" customHeight="1">
+    <row r="575" hidden="1" ht="60" customHeight="1">
       <c r="A575" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44863,7 +44862,7 @@
         </is>
       </c>
     </row>
-    <row r="576" ht="45" customHeight="1">
+    <row r="576" hidden="1" ht="45" customHeight="1">
       <c r="A576" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -44935,7 +44934,7 @@
         </is>
       </c>
     </row>
-    <row r="577" ht="75" customHeight="1">
+    <row r="577" hidden="1" ht="75" customHeight="1">
       <c r="A577" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45007,7 +45006,7 @@
         </is>
       </c>
     </row>
-    <row r="578" ht="60" customHeight="1">
+    <row r="578" hidden="1" ht="60" customHeight="1">
       <c r="A578" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45077,7 +45076,7 @@
         </is>
       </c>
     </row>
-    <row r="579" ht="75" customHeight="1">
+    <row r="579" hidden="1" ht="75" customHeight="1">
       <c r="A579" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45147,7 +45146,7 @@
         </is>
       </c>
     </row>
-    <row r="580" ht="60" customHeight="1">
+    <row r="580" hidden="1" ht="60" customHeight="1">
       <c r="A580" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45219,7 +45218,7 @@
         </is>
       </c>
     </row>
-    <row r="581" ht="60" customHeight="1">
+    <row r="581" hidden="1" ht="60" customHeight="1">
       <c r="A581" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45291,7 +45290,7 @@
         </is>
       </c>
     </row>
-    <row r="582" ht="60" customHeight="1">
+    <row r="582" hidden="1" ht="60" customHeight="1">
       <c r="A582" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45359,7 +45358,7 @@
         </is>
       </c>
     </row>
-    <row r="583" ht="60" customHeight="1">
+    <row r="583" hidden="1" ht="60" customHeight="1">
       <c r="A583" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45429,7 +45428,7 @@
         </is>
       </c>
     </row>
-    <row r="584" ht="60" customHeight="1">
+    <row r="584" hidden="1" ht="60" customHeight="1">
       <c r="A584" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45499,7 +45498,7 @@
         </is>
       </c>
     </row>
-    <row r="585" ht="60" customHeight="1">
+    <row r="585" hidden="1" ht="60" customHeight="1">
       <c r="A585" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45569,7 +45568,7 @@
         </is>
       </c>
     </row>
-    <row r="586" ht="60" customHeight="1">
+    <row r="586" hidden="1" ht="60" customHeight="1">
       <c r="A586" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45639,7 +45638,7 @@
         </is>
       </c>
     </row>
-    <row r="587" ht="45" customHeight="1">
+    <row r="587" hidden="1" ht="45" customHeight="1">
       <c r="A587" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45709,7 +45708,7 @@
         </is>
       </c>
     </row>
-    <row r="588" ht="60" customHeight="1">
+    <row r="588" hidden="1" ht="60" customHeight="1">
       <c r="A588" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45779,7 +45778,7 @@
         </is>
       </c>
     </row>
-    <row r="589" ht="45" customHeight="1">
+    <row r="589" hidden="1" ht="45" customHeight="1">
       <c r="A589" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45849,7 +45848,7 @@
         </is>
       </c>
     </row>
-    <row r="590" ht="60" customHeight="1">
+    <row r="590" hidden="1" ht="60" customHeight="1">
       <c r="A590" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -45975,7 +45974,7 @@
       <c r="Q592" s="22" t="n"/>
       <c r="R592" s="22" t="n"/>
     </row>
-    <row r="593" ht="60" customHeight="1">
+    <row r="593" hidden="1" ht="60" customHeight="1">
       <c r="A593" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46046,7 +46045,7 @@
       <c r="T593" s="4" t="n"/>
       <c r="U593" s="4" t="n"/>
     </row>
-    <row r="594" ht="45" customHeight="1">
+    <row r="594" hidden="1" ht="45" customHeight="1">
       <c r="A594" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46117,7 +46116,7 @@
       <c r="T594" s="4" t="n"/>
       <c r="U594" s="4" t="n"/>
     </row>
-    <row r="595" ht="105" customHeight="1">
+    <row r="595" hidden="1" ht="105" customHeight="1">
       <c r="A595" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46184,7 +46183,7 @@
       <c r="T595" s="4" t="n"/>
       <c r="U595" s="4" t="n"/>
     </row>
-    <row r="596" ht="90" customHeight="1">
+    <row r="596" hidden="1" ht="90" customHeight="1">
       <c r="A596" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46255,7 +46254,7 @@
       <c r="T596" s="4" t="n"/>
       <c r="U596" s="4" t="n"/>
     </row>
-    <row r="597" ht="60" customHeight="1">
+    <row r="597" hidden="1" ht="60" customHeight="1">
       <c r="A597" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46326,7 +46325,7 @@
       <c r="T597" s="4" t="n"/>
       <c r="U597" s="4" t="n"/>
     </row>
-    <row r="598" ht="75" customHeight="1">
+    <row r="598" hidden="1" ht="75" customHeight="1">
       <c r="A598" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46401,7 +46400,7 @@
       <c r="T598" s="4" t="n"/>
       <c r="U598" s="4" t="n"/>
     </row>
-    <row r="599" ht="60" customHeight="1">
+    <row r="599" hidden="1" ht="60" customHeight="1">
       <c r="A599" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46476,7 +46475,7 @@
       <c r="T599" s="4" t="n"/>
       <c r="U599" s="4" t="n"/>
     </row>
-    <row r="600" ht="45" customHeight="1">
+    <row r="600" hidden="1" ht="45" customHeight="1">
       <c r="A600" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46551,7 +46550,7 @@
       <c r="T600" s="4" t="n"/>
       <c r="U600" s="4" t="n"/>
     </row>
-    <row r="601" ht="45" customHeight="1">
+    <row r="601" hidden="1" ht="45" customHeight="1">
       <c r="A601" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46622,7 +46621,7 @@
       <c r="T601" s="4" t="n"/>
       <c r="U601" s="4" t="n"/>
     </row>
-    <row r="602" ht="30" customHeight="1">
+    <row r="602" hidden="1" ht="30" customHeight="1">
       <c r="A602" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46689,7 +46688,7 @@
       <c r="T602" s="4" t="n"/>
       <c r="U602" s="4" t="n"/>
     </row>
-    <row r="603" ht="30" customHeight="1">
+    <row r="603" hidden="1" ht="30" customHeight="1">
       <c r="A603" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46756,7 +46755,7 @@
       <c r="T603" s="4" t="n"/>
       <c r="U603" s="4" t="n"/>
     </row>
-    <row r="604" ht="30" customHeight="1">
+    <row r="604" hidden="1" ht="30" customHeight="1">
       <c r="A604" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46823,7 +46822,7 @@
       <c r="T604" s="4" t="n"/>
       <c r="U604" s="4" t="n"/>
     </row>
-    <row r="605" ht="30" customHeight="1">
+    <row r="605" hidden="1" ht="30" customHeight="1">
       <c r="A605" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46890,7 +46889,7 @@
       <c r="T605" s="4" t="n"/>
       <c r="U605" s="4" t="n"/>
     </row>
-    <row r="606" ht="45" customHeight="1">
+    <row r="606" hidden="1" ht="45" customHeight="1">
       <c r="A606" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -46957,7 +46956,7 @@
       <c r="T606" s="4" t="n"/>
       <c r="U606" s="4" t="n"/>
     </row>
-    <row r="607" ht="105" customHeight="1">
+    <row r="607" hidden="1" ht="105" customHeight="1">
       <c r="A607" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -47024,7 +47023,7 @@
       <c r="T607" s="4" t="n"/>
       <c r="U607" s="4" t="n"/>
     </row>
-    <row r="608" ht="30" customHeight="1">
+    <row r="608" hidden="1" ht="30" customHeight="1">
       <c r="A608" s="8" t="inlineStr">
         <is>
           <t>TTP</t>
@@ -48288,17 +48287,17 @@
       </c>
       <c r="C625" s="3" t="inlineStr">
         <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D625" s="6" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="E625" s="6" t="inlineStr">
+        <is>
           <t>1000</t>
-        </is>
-      </c>
-      <c r="D625" s="6" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="E625" s="6" t="inlineStr">
-        <is>
-          <t>2200</t>
         </is>
       </c>
       <c r="F625" s="15" t="inlineStr">
@@ -48360,17 +48359,17 @@
       </c>
       <c r="C626" s="7" t="inlineStr">
         <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="D626" s="7" t="inlineStr">
+        <is>
           <t>5000</t>
         </is>
       </c>
-      <c r="D626" s="7" t="inlineStr">
-        <is>
-          <t>9000</t>
-        </is>
-      </c>
       <c r="E626" s="7" t="inlineStr">
         <is>
-          <t>7000</t>
+          <t>3200</t>
         </is>
       </c>
       <c r="F626" s="31" t="inlineStr">
@@ -48432,17 +48431,17 @@
       </c>
       <c r="C627" s="6" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="D627" s="6" t="inlineStr">
         <is>
-          <t>13000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="E627" s="6" t="inlineStr">
         <is>
-          <t>11000</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="F627" s="15" t="inlineStr">
@@ -48504,7 +48503,7 @@
       </c>
       <c r="C628" s="7" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="D628" s="7" t="inlineStr">
@@ -48514,7 +48513,7 @@
       </c>
       <c r="E628" s="7" t="inlineStr">
         <is>
-          <t>12700</t>
+          <t>8500</t>
         </is>
       </c>
       <c r="F628" s="31" t="inlineStr">
@@ -48576,17 +48575,17 @@
       </c>
       <c r="C629" s="6" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="D629" s="6" t="inlineStr">
         <is>
-          <t>17000</t>
+          <t>20000</t>
         </is>
       </c>
       <c r="E629" s="6" t="inlineStr">
         <is>
-          <t>19300</t>
+          <t>14900</t>
         </is>
       </c>
       <c r="F629" s="15" t="inlineStr">
@@ -51098,16 +51097,14 @@
           <t>0056</t>
         </is>
       </c>
-      <c r="C664" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C664" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D664" s="11" t="n">
         <v>2100</v>
       </c>
       <c r="E664" s="11" t="n">
-        <v>100</v>
+        <v>1550</v>
       </c>
       <c r="F664" s="15" t="inlineStr">
         <is>
@@ -51166,16 +51163,14 @@
           <t>0057</t>
         </is>
       </c>
-      <c r="C665" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C665" s="3" t="n">
+        <v>-10000</v>
       </c>
       <c r="D665" s="11" t="n">
-        <v>2100</v>
+        <v>10000</v>
       </c>
       <c r="E665" s="11" t="n">
-        <v>100</v>
+        <v>980</v>
       </c>
       <c r="F665" s="15" t="inlineStr">
         <is>
@@ -51304,16 +51299,14 @@
           <t>0059</t>
         </is>
       </c>
-      <c r="C667" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C667" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D667" s="11" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="E667" s="11" t="n">
-        <v>200</v>
+        <v>800</v>
       </c>
       <c r="F667" s="15" t="inlineStr">
         <is>
@@ -51372,16 +51365,14 @@
           <t>0060</t>
         </is>
       </c>
-      <c r="C668" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C668" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D668" s="11" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="E668" s="11" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="F668" s="15" t="inlineStr">
         <is>
@@ -51440,13 +51431,11 @@
           <t>0061</t>
         </is>
       </c>
-      <c r="C669" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C669" s="3" t="n">
+        <v>-200</v>
       </c>
       <c r="D669" s="11" t="n">
-        <v>1100</v>
+        <v>650</v>
       </c>
       <c r="E669" s="11" t="n">
         <v>300</v>
@@ -51508,16 +51497,14 @@
           <t>0062</t>
         </is>
       </c>
-      <c r="C670" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C670" s="3" t="n">
+        <v>-200</v>
       </c>
       <c r="D670" s="11" t="n">
-        <v>1100</v>
+        <v>650</v>
       </c>
       <c r="E670" s="11" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="F670" s="15" t="inlineStr">
         <is>
@@ -51576,16 +51563,14 @@
           <t>0063</t>
         </is>
       </c>
-      <c r="C671" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C671" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="D671" s="11" t="n">
-        <v>1100</v>
+        <v>910</v>
       </c>
       <c r="E671" s="11" t="n">
-        <v>600</v>
+        <v>910</v>
       </c>
       <c r="F671" s="15" t="inlineStr">
         <is>
@@ -51644,16 +51629,14 @@
           <t>0064</t>
         </is>
       </c>
-      <c r="C672" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C672" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="D672" s="11" t="n">
-        <v>1100</v>
+        <v>910</v>
       </c>
       <c r="E672" s="11" t="n">
-        <v>500</v>
+        <v>910</v>
       </c>
       <c r="F672" s="15" t="inlineStr">
         <is>
@@ -51813,18 +51796,14 @@
       </c>
       <c r="C675" s="46" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D675" s="12" t="inlineStr">
-        <is>
-          <t>30000</t>
-        </is>
-      </c>
-      <c r="E675" s="12" t="inlineStr">
-        <is>
-          <t>8000</t>
-        </is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="D675" s="12" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E675" s="12" t="n">
+        <v>9600</v>
       </c>
       <c r="F675" s="29" t="inlineStr">
         <is>
@@ -51875,7 +51854,7 @@
       <c r="T675" s="4" t="n"/>
       <c r="U675" s="4" t="n"/>
     </row>
-    <row r="676" ht="345" customHeight="1">
+    <row r="676" hidden="1" ht="345" customHeight="1">
       <c r="A676" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -51963,7 +51942,7 @@
         </is>
       </c>
     </row>
-    <row r="677" ht="150" customHeight="1">
+    <row r="677" hidden="1" ht="150" customHeight="1">
       <c r="A677" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52037,7 +52016,7 @@
         </is>
       </c>
     </row>
-    <row r="678" ht="120" customHeight="1">
+    <row r="678" hidden="1" ht="120" customHeight="1">
       <c r="A678" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52111,7 +52090,7 @@
         </is>
       </c>
     </row>
-    <row r="679" ht="90" customHeight="1">
+    <row r="679" hidden="1" ht="90" customHeight="1">
       <c r="A679" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52179,7 +52158,7 @@
         </is>
       </c>
     </row>
-    <row r="680" ht="90" customHeight="1">
+    <row r="680" hidden="1" ht="90" customHeight="1">
       <c r="A680" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52247,7 +52226,7 @@
         </is>
       </c>
     </row>
-    <row r="681" ht="90" customHeight="1">
+    <row r="681" hidden="1" ht="90" customHeight="1">
       <c r="A681" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52315,7 +52294,7 @@
         </is>
       </c>
     </row>
-    <row r="682" ht="90" customHeight="1">
+    <row r="682" hidden="1" ht="90" customHeight="1">
       <c r="A682" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52383,7 +52362,7 @@
         </is>
       </c>
     </row>
-    <row r="683" ht="90" customHeight="1">
+    <row r="683" hidden="1" ht="90" customHeight="1">
       <c r="A683" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52451,7 +52430,7 @@
         </is>
       </c>
     </row>
-    <row r="684" ht="90" customHeight="1">
+    <row r="684" hidden="1" ht="90" customHeight="1">
       <c r="A684" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52519,7 +52498,7 @@
         </is>
       </c>
     </row>
-    <row r="685" ht="30" customHeight="1">
+    <row r="685" hidden="1" ht="30" customHeight="1">
       <c r="A685" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52587,7 +52566,7 @@
         </is>
       </c>
     </row>
-    <row r="686" ht="90" customHeight="1">
+    <row r="686" hidden="1" ht="90" customHeight="1">
       <c r="A686" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52598,16 +52577,14 @@
           <t>0011</t>
         </is>
       </c>
-      <c r="C686" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C686" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D686" s="11" t="n">
         <v>2100</v>
       </c>
       <c r="E686" s="11" t="n">
-        <v>100</v>
+        <v>1550</v>
       </c>
       <c r="F686" s="15" t="inlineStr">
         <is>
@@ -52655,7 +52632,7 @@
         </is>
       </c>
     </row>
-    <row r="687" ht="90" customHeight="1">
+    <row r="687" hidden="1" ht="90" customHeight="1">
       <c r="A687" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52666,16 +52643,14 @@
           <t>0012</t>
         </is>
       </c>
-      <c r="C687" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C687" s="3" t="n">
+        <v>-10000</v>
       </c>
       <c r="D687" s="11" t="n">
-        <v>1100</v>
+        <v>10000</v>
       </c>
       <c r="E687" s="11" t="n">
-        <v>200</v>
+        <v>980</v>
       </c>
       <c r="F687" s="15" t="inlineStr">
         <is>
@@ -52723,7 +52698,7 @@
         </is>
       </c>
     </row>
-    <row r="688" ht="90" customHeight="1">
+    <row r="688" hidden="1" ht="90" customHeight="1">
       <c r="A688" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52734,13 +52709,11 @@
           <t>0013</t>
         </is>
       </c>
-      <c r="C688" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C688" s="3" t="n">
+        <v>-200</v>
       </c>
       <c r="D688" s="11" t="n">
-        <v>1100</v>
+        <v>650</v>
       </c>
       <c r="E688" s="11" t="n">
         <v>300</v>
@@ -52791,7 +52764,7 @@
         </is>
       </c>
     </row>
-    <row r="689" ht="30" customHeight="1">
+    <row r="689" hidden="1" ht="30" customHeight="1">
       <c r="A689" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52802,16 +52775,14 @@
           <t>0014</t>
         </is>
       </c>
-      <c r="C689" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C689" s="3" t="n">
+        <v>-200</v>
       </c>
       <c r="D689" s="11" t="n">
-        <v>1100</v>
+        <v>650</v>
       </c>
       <c r="E689" s="11" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="F689" s="15" t="inlineStr">
         <is>
@@ -52859,7 +52830,7 @@
         </is>
       </c>
     </row>
-    <row r="690" ht="30" customHeight="1">
+    <row r="690" hidden="1" ht="30" customHeight="1">
       <c r="A690" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52870,16 +52841,14 @@
           <t>0015</t>
         </is>
       </c>
-      <c r="C690" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C690" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="D690" s="11" t="n">
-        <v>1100</v>
+        <v>910</v>
       </c>
       <c r="E690" s="11" t="n">
-        <v>500</v>
+        <v>910</v>
       </c>
       <c r="F690" s="15" t="inlineStr">
         <is>
@@ -52927,7 +52896,7 @@
         </is>
       </c>
     </row>
-    <row r="691" ht="30" customHeight="1">
+    <row r="691" hidden="1" ht="30" customHeight="1">
       <c r="A691" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -52938,16 +52907,14 @@
           <t>0016</t>
         </is>
       </c>
-      <c r="C691" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C691" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="D691" s="11" t="n">
-        <v>1100</v>
+        <v>910</v>
       </c>
       <c r="E691" s="11" t="n">
-        <v>600</v>
+        <v>910</v>
       </c>
       <c r="F691" s="15" t="inlineStr">
         <is>
@@ -52995,7 +52962,7 @@
         </is>
       </c>
     </row>
-    <row r="692" ht="30" customHeight="1">
+    <row r="692" hidden="1" ht="30" customHeight="1">
       <c r="A692" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53006,16 +52973,14 @@
           <t>0017</t>
         </is>
       </c>
-      <c r="C692" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C692" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D692" s="11" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="E692" s="11" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="F692" s="15" t="inlineStr">
         <is>
@@ -53063,7 +53028,7 @@
         </is>
       </c>
     </row>
-    <row r="693" ht="90" customHeight="1">
+    <row r="693" hidden="1" ht="90" customHeight="1">
       <c r="A693" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53131,7 +53096,7 @@
         </is>
       </c>
     </row>
-    <row r="694" ht="90" customHeight="1">
+    <row r="694" hidden="1" ht="90" customHeight="1">
       <c r="A694" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53197,7 +53162,7 @@
         </is>
       </c>
     </row>
-    <row r="695" ht="90" customHeight="1">
+    <row r="695" hidden="1" ht="90" customHeight="1">
       <c r="A695" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53263,7 +53228,7 @@
         </is>
       </c>
     </row>
-    <row r="696" ht="90" customHeight="1">
+    <row r="696" hidden="1" ht="90" customHeight="1">
       <c r="A696" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53329,7 +53294,7 @@
         </is>
       </c>
     </row>
-    <row r="697" ht="409.5" customHeight="1">
+    <row r="697" hidden="1" ht="409.5" customHeight="1">
       <c r="A697" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53429,7 +53394,7 @@
         </is>
       </c>
     </row>
-    <row r="698" ht="409.5" customHeight="1">
+    <row r="698" hidden="1" ht="409.5" customHeight="1">
       <c r="A698" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53528,7 +53493,7 @@
         </is>
       </c>
     </row>
-    <row r="699" ht="409.5" customHeight="1">
+    <row r="699" hidden="1" ht="409.5" customHeight="1">
       <c r="A699" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53628,7 +53593,7 @@
         </is>
       </c>
     </row>
-    <row r="700" ht="409.5" customHeight="1">
+    <row r="700" hidden="1" ht="409.5" customHeight="1">
       <c r="A700" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53728,7 +53693,7 @@
         </is>
       </c>
     </row>
-    <row r="701" ht="105" customHeight="1">
+    <row r="701" hidden="1" ht="105" customHeight="1">
       <c r="A701" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53802,7 +53767,7 @@
         </is>
       </c>
     </row>
-    <row r="702" ht="90" customHeight="1">
+    <row r="702" hidden="1" ht="90" customHeight="1">
       <c r="A702" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53875,7 +53840,7 @@
         </is>
       </c>
     </row>
-    <row r="703" ht="135" customHeight="1">
+    <row r="703" hidden="1" ht="135" customHeight="1">
       <c r="A703" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -53943,7 +53908,7 @@
         </is>
       </c>
     </row>
-    <row r="704" ht="60" customHeight="1">
+    <row r="704" hidden="1" ht="60" customHeight="1">
       <c r="A704" s="29" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -54010,7 +53975,7 @@
       <c r="T704" s="4" t="n"/>
       <c r="U704" s="4" t="n"/>
     </row>
-    <row r="705" ht="60" customHeight="1">
+    <row r="705" hidden="1" ht="60" customHeight="1">
       <c r="A705" s="29" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -54080,7 +54045,7 @@
       <c r="T705" s="4" t="n"/>
       <c r="U705" s="4" t="n"/>
     </row>
-    <row r="706" ht="90" customHeight="1">
+    <row r="706" hidden="1" ht="90" customHeight="1">
       <c r="A706" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -54150,7 +54115,7 @@
         </is>
       </c>
     </row>
-    <row r="707" ht="90" customHeight="1">
+    <row r="707" hidden="1" ht="90" customHeight="1">
       <c r="A707" s="15" t="inlineStr">
         <is>
           <t>MAS</t>
@@ -54161,16 +54126,14 @@
           <t>0032</t>
         </is>
       </c>
-      <c r="C707" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C707" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D707" s="11" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="E707" s="11" t="n">
-        <v>200</v>
+        <v>800</v>
       </c>
       <c r="F707" s="15" t="inlineStr">
         <is>
@@ -54426,7 +54389,7 @@
       <c r="Q712" s="22" t="n"/>
       <c r="R712" s="22" t="n"/>
     </row>
-    <row r="713" hidden="1" ht="45" customHeight="1">
+    <row r="713" ht="45" customHeight="1">
       <c r="A713" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54503,7 +54466,7 @@
         </is>
       </c>
     </row>
-    <row r="714" hidden="1" ht="30" customHeight="1">
+    <row r="714" ht="30" customHeight="1">
       <c r="A714" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54579,7 +54542,7 @@
         </is>
       </c>
     </row>
-    <row r="715" hidden="1" ht="90" customHeight="1">
+    <row r="715" ht="90" customHeight="1">
       <c r="A715" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54655,7 +54618,7 @@
         </is>
       </c>
     </row>
-    <row r="716" hidden="1" ht="45" customHeight="1">
+    <row r="716" ht="45" customHeight="1">
       <c r="A716" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54666,10 +54629,8 @@
           <t>0004</t>
         </is>
       </c>
-      <c r="C716" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C716" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D716" s="11" t="n">
         <v>1</v>
@@ -54731,7 +54692,7 @@
         </is>
       </c>
     </row>
-    <row r="717" hidden="1" ht="45" customHeight="1">
+    <row r="717" ht="45" customHeight="1">
       <c r="A717" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54742,10 +54703,8 @@
           <t>0005</t>
         </is>
       </c>
-      <c r="C717" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C717" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D717" s="11" t="n">
         <v>1</v>
@@ -54807,7 +54766,7 @@
         </is>
       </c>
     </row>
-    <row r="718" hidden="1" ht="45" customHeight="1">
+    <row r="718" ht="45" customHeight="1">
       <c r="A718" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54818,10 +54777,8 @@
           <t>0006</t>
         </is>
       </c>
-      <c r="C718" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C718" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D718" s="11" t="n">
         <v>1</v>
@@ -54883,7 +54840,7 @@
         </is>
       </c>
     </row>
-    <row r="719" hidden="1" ht="45" customHeight="1">
+    <row r="719" ht="45" customHeight="1">
       <c r="A719" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54894,10 +54851,8 @@
           <t>0007</t>
         </is>
       </c>
-      <c r="C719" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C719" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D719" s="11" t="n">
         <v>1</v>
@@ -54959,7 +54914,7 @@
         </is>
       </c>
     </row>
-    <row r="720" hidden="1" ht="45" customHeight="1">
+    <row r="720" ht="45" customHeight="1">
       <c r="A720" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -54970,10 +54925,8 @@
           <t>0008</t>
         </is>
       </c>
-      <c r="C720" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C720" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D720" s="11" t="n">
         <v>1</v>
@@ -55035,7 +54988,7 @@
         </is>
       </c>
     </row>
-    <row r="721" hidden="1" ht="45" customHeight="1">
+    <row r="721" ht="45" customHeight="1">
       <c r="A721" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55046,10 +54999,8 @@
           <t>0009</t>
         </is>
       </c>
-      <c r="C721" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C721" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D721" s="11" t="n">
         <v>1</v>
@@ -55111,7 +55062,7 @@
         </is>
       </c>
     </row>
-    <row r="722" hidden="1" ht="45" customHeight="1">
+    <row r="722" ht="45" customHeight="1">
       <c r="A722" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55122,10 +55073,8 @@
           <t>0010</t>
         </is>
       </c>
-      <c r="C722" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C722" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D722" s="11" t="n">
         <v>1</v>
@@ -55187,7 +55136,7 @@
         </is>
       </c>
     </row>
-    <row r="723" hidden="1" ht="90" customHeight="1">
+    <row r="723" ht="90" customHeight="1">
       <c r="A723" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55263,7 +55212,7 @@
         </is>
       </c>
     </row>
-    <row r="724" hidden="1" ht="90" customHeight="1">
+    <row r="724" ht="90" customHeight="1">
       <c r="A724" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55339,7 +55288,7 @@
         </is>
       </c>
     </row>
-    <row r="725" hidden="1" ht="90" customHeight="1">
+    <row r="725" ht="90" customHeight="1">
       <c r="A725" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55415,7 +55364,7 @@
         </is>
       </c>
     </row>
-    <row r="726" hidden="1" ht="90" customHeight="1">
+    <row r="726" ht="90" customHeight="1">
       <c r="A726" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55491,7 +55440,7 @@
         </is>
       </c>
     </row>
-    <row r="727" hidden="1" ht="30" customHeight="1">
+    <row r="727" ht="30" customHeight="1">
       <c r="A727" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55567,7 +55516,7 @@
         </is>
       </c>
     </row>
-    <row r="728" hidden="1" ht="90" customHeight="1">
+    <row r="728" ht="90" customHeight="1">
       <c r="A728" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55643,7 +55592,7 @@
         </is>
       </c>
     </row>
-    <row r="729" hidden="1" ht="90" customHeight="1">
+    <row r="729" ht="90" customHeight="1">
       <c r="A729" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55719,7 +55668,7 @@
         </is>
       </c>
     </row>
-    <row r="730" hidden="1" ht="45" customHeight="1">
+    <row r="730" ht="45" customHeight="1">
       <c r="A730" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55795,7 +55744,7 @@
         </is>
       </c>
     </row>
-    <row r="731" hidden="1" ht="90" customHeight="1">
+    <row r="731" ht="90" customHeight="1">
       <c r="A731" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55871,7 +55820,7 @@
         </is>
       </c>
     </row>
-    <row r="732" hidden="1" ht="90" customHeight="1">
+    <row r="732" ht="90" customHeight="1">
       <c r="A732" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -55947,7 +55896,7 @@
         </is>
       </c>
     </row>
-    <row r="733" hidden="1" ht="30" customHeight="1">
+    <row r="733" ht="30" customHeight="1">
       <c r="A733" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56023,7 +55972,7 @@
         </is>
       </c>
     </row>
-    <row r="734" hidden="1" ht="30" customHeight="1">
+    <row r="734" ht="30" customHeight="1">
       <c r="A734" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56099,7 +56048,7 @@
         </is>
       </c>
     </row>
-    <row r="735" hidden="1" ht="45" customHeight="1">
+    <row r="735" ht="45" customHeight="1">
       <c r="A735" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56176,7 +56125,7 @@
         </is>
       </c>
     </row>
-    <row r="736" hidden="1" ht="90" customHeight="1">
+    <row r="736" ht="90" customHeight="1">
       <c r="A736" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56252,7 +56201,7 @@
         </is>
       </c>
     </row>
-    <row r="737" hidden="1" ht="90" customHeight="1">
+    <row r="737" ht="90" customHeight="1">
       <c r="A737" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56328,7 +56277,7 @@
         </is>
       </c>
     </row>
-    <row r="738" hidden="1" ht="90" customHeight="1">
+    <row r="738" ht="90" customHeight="1">
       <c r="A738" s="15" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56404,7 +56353,7 @@
         </is>
       </c>
     </row>
-    <row r="739" hidden="1" ht="30" customHeight="1">
+    <row r="739" ht="30" customHeight="1">
       <c r="A739" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56481,7 +56430,7 @@
         </is>
       </c>
     </row>
-    <row r="740" hidden="1" ht="30" customHeight="1">
+    <row r="740" ht="30" customHeight="1">
       <c r="A740" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56557,7 +56506,7 @@
         </is>
       </c>
     </row>
-    <row r="741" hidden="1" ht="75" customHeight="1">
+    <row r="741" ht="75" customHeight="1">
       <c r="A741" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56633,7 +56582,7 @@
         </is>
       </c>
     </row>
-    <row r="742" hidden="1" ht="30" customHeight="1">
+    <row r="742" ht="30" customHeight="1">
       <c r="A742" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56709,7 +56658,7 @@
         </is>
       </c>
     </row>
-    <row r="743" hidden="1" ht="30" customHeight="1">
+    <row r="743" ht="30" customHeight="1">
       <c r="A743" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56788,7 +56737,7 @@
       <c r="T743" s="4" t="n"/>
       <c r="U743" s="4" t="n"/>
     </row>
-    <row r="744" hidden="1" ht="75" customHeight="1">
+    <row r="744" ht="75" customHeight="1">
       <c r="A744" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56864,7 +56813,7 @@
         </is>
       </c>
     </row>
-    <row r="745" hidden="1" ht="30" customHeight="1">
+    <row r="745" ht="30" customHeight="1">
       <c r="A745" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -56940,7 +56889,7 @@
         </is>
       </c>
     </row>
-    <row r="746" hidden="1" ht="30" customHeight="1">
+    <row r="746" ht="30" customHeight="1">
       <c r="A746" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57016,7 +56965,7 @@
         </is>
       </c>
     </row>
-    <row r="747" hidden="1" ht="30" customHeight="1">
+    <row r="747" ht="30" customHeight="1">
       <c r="A747" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57095,7 +57044,7 @@
       <c r="T747" s="4" t="n"/>
       <c r="U747" s="4" t="n"/>
     </row>
-    <row r="748" hidden="1" ht="90" customHeight="1">
+    <row r="748" ht="90" customHeight="1">
       <c r="A748" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57171,7 +57120,7 @@
         </is>
       </c>
     </row>
-    <row r="749" hidden="1" ht="90" customHeight="1">
+    <row r="749" ht="90" customHeight="1">
       <c r="A749" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57247,7 +57196,7 @@
         </is>
       </c>
     </row>
-    <row r="750" hidden="1" ht="90" customHeight="1">
+    <row r="750" ht="90" customHeight="1">
       <c r="A750" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57319,7 +57268,7 @@
         </is>
       </c>
     </row>
-    <row r="751" hidden="1" ht="90" customHeight="1">
+    <row r="751" ht="90" customHeight="1">
       <c r="A751" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57391,7 +57340,7 @@
         </is>
       </c>
     </row>
-    <row r="752" hidden="1" ht="90" customHeight="1">
+    <row r="752" ht="90" customHeight="1">
       <c r="A752" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57463,7 +57412,7 @@
         </is>
       </c>
     </row>
-    <row r="753" hidden="1" ht="30" customHeight="1">
+    <row r="753" ht="30" customHeight="1">
       <c r="A753" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57535,7 +57484,7 @@
         </is>
       </c>
     </row>
-    <row r="754" hidden="1" ht="90" customHeight="1">
+    <row r="754" ht="90" customHeight="1">
       <c r="A754" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57607,7 +57556,7 @@
         </is>
       </c>
     </row>
-    <row r="755" hidden="1" ht="30" customHeight="1">
+    <row r="755" ht="30" customHeight="1">
       <c r="A755" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57683,7 +57632,7 @@
         </is>
       </c>
     </row>
-    <row r="756" hidden="1" ht="45" customHeight="1">
+    <row r="756" ht="45" customHeight="1">
       <c r="A756" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57755,7 +57704,7 @@
         </is>
       </c>
     </row>
-    <row r="757" hidden="1" ht="45" customHeight="1">
+    <row r="757" ht="45" customHeight="1">
       <c r="A757" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57831,7 +57780,7 @@
         </is>
       </c>
     </row>
-    <row r="758" hidden="1" ht="150" customHeight="1">
+    <row r="758" ht="150" customHeight="1">
       <c r="A758" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57842,10 +57791,8 @@
           <t>0046</t>
         </is>
       </c>
-      <c r="C758" s="43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C758" s="43" t="n">
+        <v>0</v>
       </c>
       <c r="D758" s="11" t="n">
         <v>1</v>
@@ -57907,7 +57854,7 @@
         </is>
       </c>
     </row>
-    <row r="759" hidden="1" ht="120" customHeight="1">
+    <row r="759" ht="120" customHeight="1">
       <c r="A759" s="10" t="inlineStr">
         <is>
           <t>MAE</t>
@@ -57918,10 +57865,8 @@
           <t>0047</t>
         </is>
       </c>
-      <c r="C759" s="43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C759" s="43" t="n">
+        <v>0</v>
       </c>
       <c r="D759" s="11" t="n">
         <v>1</v>
@@ -58255,7 +58200,7 @@
       <c r="T763" s="4" t="n"/>
       <c r="U763" s="4" t="n"/>
     </row>
-    <row r="764" hidden="1">
+    <row r="764" hidden="1" ht="135" customHeight="1">
       <c r="A764" s="10" t="inlineStr">
         <is>
           <t>MAC</t>
@@ -58324,7 +58269,7 @@
       <c r="T764" s="4" t="n"/>
       <c r="U764" s="4" t="n"/>
     </row>
-    <row r="765" hidden="1">
+    <row r="765" hidden="1" ht="135" customHeight="1">
       <c r="A765" s="10" t="inlineStr">
         <is>
           <t>MAC</t>
@@ -58708,4 +58653,296 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a32518fee107c04aa9bd7948c0d3f18">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e97db55af52189d57b3fce0d0bdbaea8" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
+    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19930CF4-2EE6-43B1-B275-7A602E166EFE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64468085-42FE-47F1-A7E2-4F975A580B50}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0AB6D09-120D-4712-8811-F293FA38E8C9}"/>
 </file>
</xml_diff>

<commit_message>
Enforce Motor 3 stop tolerance
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="rng_Lieferanten">#REF!</definedName>
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U780"/>
+  <dimension ref="A1:U781"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="16.140625" bestFit="1" customWidth="1" style="13" min="1" max="1"/>
@@ -57928,22 +57928,22 @@
         </is>
       </c>
     </row>
-    <row r="760" hidden="1" ht="135" customHeight="1">
+    <row r="760" hidden="1" ht="120" customHeight="1">
       <c r="A760" s="10" t="inlineStr">
         <is>
-          <t>MAC</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="B760" s="8" t="inlineStr">
         <is>
-          <t>0001</t>
+          <t>0048</t>
         </is>
       </c>
       <c r="C760" s="46" t="n">
         <v>0</v>
       </c>
       <c r="D760" s="12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E760" s="12" t="n">
         <v>0</v>
@@ -57952,22 +57952,22 @@
       <c r="G760" s="29" t="n"/>
       <c r="H760" s="29" t="inlineStr">
         <is>
-          <t>R/W</t>
+          <t>R</t>
         </is>
       </c>
       <c r="I760" s="29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>W</t>
         </is>
       </c>
       <c r="J760" s="29" t="inlineStr">
         <is>
-          <t>uint8</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="K760" s="29" t="inlineStr">
         <is>
-          <t>Temporaerer IBN/Test Prozessbefehl</t>
+          <t>MAE0048 Etikettenantrieb Nachpositionierung Toleranz nicht erreicht</t>
         </is>
       </c>
       <c r="L760" s="28" t="n"/>
@@ -57978,15 +57978,27 @@
       </c>
       <c r="N760" s="28" t="inlineStr">
         <is>
-          <t>0=Stop, 1=Wickler einmessen+Messfahrt, 2=Taktbetrieb, 3=Vorziehen kontinuierlich, 4=Zurueckspulen kontinuierlich</t>
-        </is>
-      </c>
-      <c r="O760" s="28" t="n"/>
-      <c r="P760" s="28" t="n"/>
-      <c r="Q760" s="28" t="n"/>
+          <t>Etikettenantrieb Nachpositionierung: Toleranz +/-0.05 mm nach 3 Versuchen nicht erreicht</t>
+        </is>
+      </c>
+      <c r="O760" s="28" t="inlineStr">
+        <is>
+          <t>Schlupf, mechanische Blockade, falsche Motoraufl?sung, Encoderabweichung oder AZD-Parameter ausserhalb des stabilen Bereichs</t>
+        </is>
+      </c>
+      <c r="P760" s="28" t="inlineStr">
+        <is>
+          <t>Mess-/Taktposition wird verworfen; Produktion oder Einrichten wird abgebrochen, weil die Druckposition nicht garantiert werden kann</t>
+        </is>
+      </c>
+      <c r="Q760" s="28" t="inlineStr">
+        <is>
+          <t>Mechanik, Bandspannung, Motoraufl?sung, Encoderwerte und AZD-Parameter pr?fen; danach Reset und erneutes Einrichten ausf?hren</t>
+        </is>
+      </c>
       <c r="R760" s="28" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe MAC0001 als temporaeren IBN-/Testbefehl von Microtom an den Raspi. Der Raspi uebersetzt diesen Wert in produktionsnahe Startkommandos fuer ESP32-PLC und Wickler. Dieser Parameter ist ausdruecklich nur fuer Inbetriebnahme/Test vorgesehen und muss spaeter entfernt oder durch produktive MAS/MAP-Ablaufbefehle ersetzt werden. Der ESP soll ihn gemaess Masterliste nicht direkt als normalen Parameter verwenden. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe MAE0048 als Stoerungsmeldung, wenn Motor 3 nach einer Mess- oder Taktposition seine Sollposition trotz maximal drei Nachpositionierungen nicht innerhalb von +/-0.05 mm erreicht. Waehrend dieser Nachpositionierung muessen Abwickler und Aufwickler stillstehen und duerfen nicht selbst nachregeln.</t>
         </is>
       </c>
       <c r="S760" s="4" t="n"/>
@@ -58001,23 +58013,19 @@
       </c>
       <c r="B761" s="8" t="inlineStr">
         <is>
-          <t>0002</t>
+          <t>0001</t>
         </is>
       </c>
       <c r="C761" s="46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D761" s="12" t="n">
-        <v>5000</v>
+        <v>4</v>
       </c>
       <c r="E761" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F761" s="29" t="inlineStr">
-        <is>
-          <t>1/10mm</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F761" s="29" t="n"/>
       <c r="G761" s="29" t="n"/>
       <c r="H761" s="29" t="inlineStr">
         <is>
@@ -58031,12 +58039,12 @@
       </c>
       <c r="J761" s="29" t="inlineStr">
         <is>
-          <t>uint16</t>
+          <t>uint8</t>
         </is>
       </c>
       <c r="K761" s="29" t="inlineStr">
         <is>
-          <t>Temporaere Takt-/Labellaenge</t>
+          <t>Temporaerer IBN/Test Prozessbefehl</t>
         </is>
       </c>
       <c r="L761" s="28" t="n"/>
@@ -58047,7 +58055,7 @@
       </c>
       <c r="N761" s="28" t="inlineStr">
         <is>
-          <t>Labelweg fuer getakteten Testbetrieb in 1/10 mm</t>
+          <t>0=Stop, 1=Wickler einmessen+Messfahrt, 2=Taktbetrieb, 3=Vorziehen kontinuierlich, 4=Zurueckspulen kontinuierlich</t>
         </is>
       </c>
       <c r="O761" s="28" t="n"/>
@@ -58055,7 +58063,7 @@
       <c r="Q761" s="28" t="n"/>
       <c r="R761" s="28" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe MAC0002 als temporaere Labellaenge bzw. Taktstrecke fuer den IBN-Test. Default 1000 bedeutet 100.0 mm. Spaeter kommt dieser Wert aus Rezept-/Formatdaten und Etiketteneinmessung, nicht mehr aus einem MAC-Testparameter. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe MAC0001 als temporaeren IBN-/Testbefehl von Microtom an den Raspi. Der Raspi uebersetzt diesen Wert in produktionsnahe Startkommandos fuer ESP32-PLC und Wickler. Dieser Parameter ist ausdruecklich nur fuer Inbetriebnahme/Test vorgesehen und muss spaeter entfernt oder durch produktive MAS/MAP-Ablaufbefehle ersetzt werden. Der ESP soll ihn gemaess Masterliste nicht direkt als normalen Parameter verwenden. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
       <c r="S761" s="4" t="n"/>
@@ -58070,21 +58078,21 @@
       </c>
       <c r="B762" s="8" t="inlineStr">
         <is>
-          <t>0003</t>
+          <t>0002</t>
         </is>
       </c>
       <c r="C762" s="46" t="n">
         <v>1</v>
       </c>
       <c r="D762" s="12" t="n">
-        <v>400</v>
+        <v>5000</v>
       </c>
       <c r="E762" s="12" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F762" s="29" t="inlineStr">
         <is>
-          <t>mm/s</t>
+          <t>1/10mm</t>
         </is>
       </c>
       <c r="G762" s="29" t="n"/>
@@ -58105,7 +58113,7 @@
       </c>
       <c r="K762" s="29" t="inlineStr">
         <is>
-          <t>Temporaere Vorzugsgeschwindigkeit</t>
+          <t>Temporaere Takt-/Labellaenge</t>
         </is>
       </c>
       <c r="L762" s="28" t="n"/>
@@ -58116,7 +58124,7 @@
       </c>
       <c r="N762" s="28" t="inlineStr">
         <is>
-          <t>Sollgeschwindigkeit fuer kontinuierlichen und getakteten IBN-Testbetrieb</t>
+          <t>Labelweg fuer getakteten Testbetrieb in 1/10 mm</t>
         </is>
       </c>
       <c r="O762" s="28" t="n"/>
@@ -58124,7 +58132,7 @@
       <c r="Q762" s="28" t="n"/>
       <c r="R762" s="28" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe MAC0003 als temporaere Vorzugsgeschwindigkeit fuer Motor 3 im IBN-Test. Wird kein neuer Wert gesetzt, verwendet der Raspi den zuletzt gespeicherten Wert. Produktiv wird die Geschwindigkeit ueber MAP0014 bzw. die Betriebsart vorgegeben. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe MAC0002 als temporaere Labellaenge bzw. Taktstrecke fuer den IBN-Test. Default 1000 bedeutet 100.0 mm. Spaeter kommt dieser Wert aus Rezept-/Formatdaten und Etiketteneinmessung, nicht mehr aus einem MAC-Testparameter. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
       <c r="S762" s="4" t="n"/>
@@ -58139,21 +58147,21 @@
       </c>
       <c r="B763" s="8" t="inlineStr">
         <is>
-          <t>0004</t>
+          <t>0003</t>
         </is>
       </c>
       <c r="C763" s="46" t="n">
         <v>1</v>
       </c>
       <c r="D763" s="12" t="n">
-        <v>6000</v>
+        <v>400</v>
       </c>
       <c r="E763" s="12" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F763" s="29" t="inlineStr">
         <is>
-          <t>mm/s2</t>
+          <t>mm/s</t>
         </is>
       </c>
       <c r="G763" s="29" t="n"/>
@@ -58174,7 +58182,7 @@
       </c>
       <c r="K763" s="29" t="inlineStr">
         <is>
-          <t>Temporaere Transport-Rampe</t>
+          <t>Temporaere Vorzugsgeschwindigkeit</t>
         </is>
       </c>
       <c r="L763" s="28" t="n"/>
@@ -58185,7 +58193,7 @@
       </c>
       <c r="N763" s="28" t="inlineStr">
         <is>
-          <t>Beschleunigung/Verzoegerung fuer Motor 3 im IBN-Testbetrieb</t>
+          <t>Sollgeschwindigkeit fuer kontinuierlichen und getakteten IBN-Testbetrieb</t>
         </is>
       </c>
       <c r="O763" s="28" t="n"/>
@@ -58193,7 +58201,7 @@
       <c r="Q763" s="28" t="n"/>
       <c r="R763" s="28" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe MAC0004 als temporaere Rampe fuer Beschleunigung und Bremsung des Etikettenantriebs im IBN-Test. Produktiv wird diese Vorgabe aus Maschinen- bzw. Formatparametern abgeleitet und darf den Etikettenschlupf nicht erhoehen. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s2. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe MAC0003 als temporaere Vorzugsgeschwindigkeit fuer Motor 3 im IBN-Test. Wird kein neuer Wert gesetzt, verwendet der Raspi den zuletzt gespeicherten Wert. Produktiv wird die Geschwindigkeit ueber MAP0014 bzw. die Betriebsart vorgegeben. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
       <c r="S763" s="4" t="n"/>
@@ -58208,21 +58216,21 @@
       </c>
       <c r="B764" s="8" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0004</t>
         </is>
       </c>
       <c r="C764" s="46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D764" s="12" t="n">
-        <v>100000</v>
+        <v>6000</v>
       </c>
       <c r="E764" s="12" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F764" s="29" t="inlineStr">
         <is>
-          <t>1/10mm</t>
+          <t>mm/s2</t>
         </is>
       </c>
       <c r="G764" s="29" t="n"/>
@@ -58238,12 +58246,12 @@
       </c>
       <c r="J764" s="29" t="inlineStr">
         <is>
-          <t>uint32</t>
+          <t>uint16</t>
         </is>
       </c>
       <c r="K764" s="29" t="inlineStr">
         <is>
-          <t>Temporaere kontinuierliche Weglaenge</t>
+          <t>Temporaere Transport-Rampe</t>
         </is>
       </c>
       <c r="L764" s="28" t="n"/>
@@ -58254,7 +58262,7 @@
       </c>
       <c r="N764" s="28" t="inlineStr">
         <is>
-          <t>Weg fuer kontinuierliches Vorziehen/Rueckspulen; 0=endlos bis Stop</t>
+          <t>Beschleunigung/Verzoegerung fuer Motor 3 im IBN-Testbetrieb</t>
         </is>
       </c>
       <c r="O764" s="28" t="n"/>
@@ -58262,7 +58270,7 @@
       <c r="Q764" s="28" t="n"/>
       <c r="R764" s="28" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe MAC0005 als temporaere Wegvorgabe fuer kontinuierliches Vorziehen oder Rueckspulen. Default 0 bedeutet endlos fahren bis MAC0001=0. Produktiv wird diese Laenge aus Ablaufzustand, Rueckspulweg oder Bedienhandlung bestimmt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe MAC0004 als temporaere Rampe fuer Beschleunigung und Bremsung des Etikettenantriebs im IBN-Test. Produktiv wird diese Vorgabe aus Maschinen- bzw. Formatparametern abgeleitet und darf den Etikettenschlupf nicht erhoehen. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s2. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
       <c r="S764" s="4" t="n"/>
@@ -58277,21 +58285,21 @@
       </c>
       <c r="B765" s="8" t="inlineStr">
         <is>
-          <t>0006</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="C765" s="46" t="n">
         <v>0</v>
       </c>
       <c r="D765" s="12" t="n">
-        <v>1000</v>
+        <v>100000</v>
       </c>
       <c r="E765" s="12" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F765" s="29" t="inlineStr">
         <is>
-          <t>Zyklen</t>
+          <t>1/10mm</t>
         </is>
       </c>
       <c r="G765" s="29" t="n"/>
@@ -58307,12 +58315,12 @@
       </c>
       <c r="J765" s="29" t="inlineStr">
         <is>
-          <t>uint16</t>
+          <t>uint32</t>
         </is>
       </c>
       <c r="K765" s="29" t="inlineStr">
         <is>
-          <t>Temporaere Taktzyklus-Anzahl</t>
+          <t>Temporaere kontinuierliche Weglaenge</t>
         </is>
       </c>
       <c r="L765" s="28" t="n"/>
@@ -58323,7 +58331,7 @@
       </c>
       <c r="N765" s="28" t="inlineStr">
         <is>
-          <t>Anzahl Takte im Testbetrieb; 0=endlos bis Stop</t>
+          <t>Weg fuer kontinuierliches Vorziehen/Rueckspulen; 0=endlos bis Stop</t>
         </is>
       </c>
       <c r="O765" s="28" t="n"/>
@@ -58331,7 +58339,7 @@
       <c r="Q765" s="28" t="n"/>
       <c r="R765" s="28" t="inlineStr">
         <is>
-          <t>KI: Ich verstehe MAC0006 als temporaere Zyklusanzahl fuer den getakteten IBN-Test. Default 20 entspricht einem kurzen Stabilitaetstest; 0 bedeutet laufender Taktbetrieb bis MAC0001=0. Spaeter wird diese Logik durch den echten Produktionsablauf und das Schieberegister ersetzt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: Zyklen. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+          <t>KI: Ich verstehe MAC0005 als temporaere Wegvorgabe fuer kontinuierliches Vorziehen oder Rueckspulen. Default 0 bedeutet endlos fahren bis MAC0001=0. Produktiv wird diese Laenge aus Ablaufzustand, Rueckspulweg oder Bedienhandlung bestimmt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
         </is>
       </c>
       <c r="S765" s="4" t="n"/>
@@ -58339,24 +58347,73 @@
       <c r="U765" s="4" t="n"/>
     </row>
     <row r="766" hidden="1">
-      <c r="A766" s="10" t="n"/>
-      <c r="B766" s="8" t="n"/>
-      <c r="C766" s="43" t="n"/>
-      <c r="D766" s="11" t="n"/>
-      <c r="E766" s="11" t="n"/>
-      <c r="F766" s="15" t="n"/>
-      <c r="G766" s="15" t="n"/>
-      <c r="H766" s="15" t="n"/>
-      <c r="I766" s="15" t="n"/>
-      <c r="J766" s="15" t="n"/>
-      <c r="K766" s="15" t="n"/>
-      <c r="L766" s="22" t="n"/>
-      <c r="M766" s="22" t="n"/>
-      <c r="N766" s="22" t="n"/>
-      <c r="O766" s="22" t="n"/>
-      <c r="P766" s="22" t="n"/>
-      <c r="Q766" s="22" t="n"/>
-      <c r="R766" s="22" t="n"/>
+      <c r="A766" s="10" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="B766" s="8" t="inlineStr">
+        <is>
+          <t>0006</t>
+        </is>
+      </c>
+      <c r="C766" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D766" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E766" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F766" s="29" t="inlineStr">
+        <is>
+          <t>Zyklen</t>
+        </is>
+      </c>
+      <c r="G766" s="29" t="n"/>
+      <c r="H766" s="29" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="I766" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J766" s="29" t="inlineStr">
+        <is>
+          <t>uint16</t>
+        </is>
+      </c>
+      <c r="K766" s="29" t="inlineStr">
+        <is>
+          <t>Temporaere Taktzyklus-Anzahl</t>
+        </is>
+      </c>
+      <c r="L766" s="28" t="n"/>
+      <c r="M766" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N766" s="28" t="inlineStr">
+        <is>
+          <t>Anzahl Takte im Testbetrieb; 0=endlos bis Stop</t>
+        </is>
+      </c>
+      <c r="O766" s="28" t="n"/>
+      <c r="P766" s="28" t="n"/>
+      <c r="Q766" s="28" t="n"/>
+      <c r="R766" s="28" t="inlineStr">
+        <is>
+          <t>KI: Ich verstehe MAC0006 als temporaere Zyklusanzahl fuer den getakteten IBN-Test. Default 20 entspricht einem kurzen Stabilitaetstest; 0 bedeutet laufender Taktbetrieb bis MAC0001=0. Spaeter wird diese Logik durch den echten Produktionsablauf und das Schieberegister ersetzt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: Zyklen. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
+        </is>
+      </c>
+      <c r="S766" s="4" t="n"/>
+      <c r="T766" s="4" t="n"/>
+      <c r="U766" s="4" t="n"/>
     </row>
     <row r="767" hidden="1">
       <c r="A767" s="10" t="n"/>
@@ -58638,6 +58695,26 @@
       <c r="Q780" s="22" t="n"/>
       <c r="R780" s="22" t="n"/>
     </row>
+    <row r="781">
+      <c r="A781" s="10" t="n"/>
+      <c r="B781" s="8" t="n"/>
+      <c r="C781" s="43" t="n"/>
+      <c r="D781" s="11" t="n"/>
+      <c r="E781" s="11" t="n"/>
+      <c r="F781" s="15" t="n"/>
+      <c r="G781" s="15" t="n"/>
+      <c r="H781" s="15" t="n"/>
+      <c r="I781" s="15" t="n"/>
+      <c r="J781" s="15" t="n"/>
+      <c r="K781" s="15" t="n"/>
+      <c r="L781" s="22" t="n"/>
+      <c r="M781" s="22" t="n"/>
+      <c r="N781" s="22" t="n"/>
+      <c r="O781" s="22" t="n"/>
+      <c r="P781" s="22" t="n"/>
+      <c r="Q781" s="22" t="n"/>
+      <c r="R781" s="22" t="n"/>
+    </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation sqref="M1:M1048576 P2:P119" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -58653,296 +58730,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a32518fee107c04aa9bd7948c0d3f18">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e97db55af52189d57b3fce0d0bdbaea8" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
-    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
-    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19930CF4-2EE6-43B1-B275-7A602E166EFE}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64468085-42FE-47F1-A7E2-4F975A580B50}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0AB6D09-120D-4712-8811-F293FA38E8C9}"/>
 </file>
</xml_diff>

<commit_message>
Remove temporary MAC commands
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U781"/>
+  <dimension ref="A1:U775"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="16.140625" bestFit="1" customWidth="1" style="13" min="1" max="1"/>
@@ -58006,414 +58006,124 @@
       <c r="U760" s="4" t="n"/>
     </row>
     <row r="761" hidden="1" ht="120" customHeight="1">
-      <c r="A761" s="10" t="inlineStr">
-        <is>
-          <t>MAC</t>
-        </is>
-      </c>
-      <c r="B761" s="8" t="inlineStr">
-        <is>
-          <t>0001</t>
-        </is>
-      </c>
-      <c r="C761" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="D761" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E761" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F761" s="29" t="n"/>
-      <c r="G761" s="29" t="n"/>
-      <c r="H761" s="29" t="inlineStr">
-        <is>
-          <t>R/W</t>
-        </is>
-      </c>
-      <c r="I761" s="29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J761" s="29" t="inlineStr">
-        <is>
-          <t>uint8</t>
-        </is>
-      </c>
-      <c r="K761" s="29" t="inlineStr">
-        <is>
-          <t>Temporaerer IBN/Test Prozessbefehl</t>
-        </is>
-      </c>
-      <c r="L761" s="28" t="n"/>
-      <c r="M761" s="28" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N761" s="28" t="inlineStr">
-        <is>
-          <t>0=Stop, 1=Wickler einmessen+Messfahrt, 2=Taktbetrieb, 3=Vorziehen kontinuierlich, 4=Zurueckspulen kontinuierlich</t>
-        </is>
-      </c>
-      <c r="O761" s="28" t="n"/>
-      <c r="P761" s="28" t="n"/>
-      <c r="Q761" s="28" t="n"/>
-      <c r="R761" s="28" t="inlineStr">
-        <is>
-          <t>KI: Ich verstehe MAC0001 als temporaeren IBN-/Testbefehl von Microtom an den Raspi. Der Raspi uebersetzt diesen Wert in produktionsnahe Startkommandos fuer ESP32-PLC und Wickler. Dieser Parameter ist ausdruecklich nur fuer Inbetriebnahme/Test vorgesehen und muss spaeter entfernt oder durch produktive MAS/MAP-Ablaufbefehle ersetzt werden. Der ESP soll ihn gemaess Masterliste nicht direkt als normalen Parameter verwenden. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-      <c r="S761" s="4" t="n"/>
-      <c r="T761" s="4" t="n"/>
-      <c r="U761" s="4" t="n"/>
+      <c r="A761" s="10" t="n"/>
+      <c r="B761" s="8" t="n"/>
+      <c r="C761" s="43" t="n"/>
+      <c r="D761" s="11" t="n"/>
+      <c r="E761" s="11" t="n"/>
+      <c r="F761" s="15" t="n"/>
+      <c r="G761" s="15" t="n"/>
+      <c r="H761" s="15" t="n"/>
+      <c r="I761" s="15" t="n"/>
+      <c r="J761" s="15" t="n"/>
+      <c r="K761" s="15" t="n"/>
+      <c r="L761" s="22" t="n"/>
+      <c r="M761" s="22" t="n"/>
+      <c r="N761" s="22" t="n"/>
+      <c r="O761" s="22" t="n"/>
+      <c r="P761" s="22" t="n"/>
+      <c r="Q761" s="22" t="n"/>
+      <c r="R761" s="22" t="n"/>
     </row>
     <row r="762" hidden="1" ht="135" customHeight="1">
-      <c r="A762" s="10" t="inlineStr">
-        <is>
-          <t>MAC</t>
-        </is>
-      </c>
-      <c r="B762" s="8" t="inlineStr">
-        <is>
-          <t>0002</t>
-        </is>
-      </c>
-      <c r="C762" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D762" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E762" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F762" s="29" t="inlineStr">
-        <is>
-          <t>1/10mm</t>
-        </is>
-      </c>
-      <c r="G762" s="29" t="n"/>
-      <c r="H762" s="29" t="inlineStr">
-        <is>
-          <t>R/W</t>
-        </is>
-      </c>
-      <c r="I762" s="29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J762" s="29" t="inlineStr">
-        <is>
-          <t>uint16</t>
-        </is>
-      </c>
-      <c r="K762" s="29" t="inlineStr">
-        <is>
-          <t>Temporaere Takt-/Labellaenge</t>
-        </is>
-      </c>
-      <c r="L762" s="28" t="n"/>
-      <c r="M762" s="28" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N762" s="28" t="inlineStr">
-        <is>
-          <t>Labelweg fuer getakteten Testbetrieb in 1/10 mm</t>
-        </is>
-      </c>
-      <c r="O762" s="28" t="n"/>
-      <c r="P762" s="28" t="n"/>
-      <c r="Q762" s="28" t="n"/>
-      <c r="R762" s="28" t="inlineStr">
-        <is>
-          <t>KI: Ich verstehe MAC0002 als temporaere Labellaenge bzw. Taktstrecke fuer den IBN-Test. Default 1000 bedeutet 100.0 mm. Spaeter kommt dieser Wert aus Rezept-/Formatdaten und Etiketteneinmessung, nicht mehr aus einem MAC-Testparameter. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-      <c r="S762" s="4" t="n"/>
-      <c r="T762" s="4" t="n"/>
-      <c r="U762" s="4" t="n"/>
+      <c r="A762" s="10" t="n"/>
+      <c r="B762" s="8" t="n"/>
+      <c r="C762" s="43" t="n"/>
+      <c r="D762" s="11" t="n"/>
+      <c r="E762" s="11" t="n"/>
+      <c r="F762" s="15" t="n"/>
+      <c r="G762" s="15" t="n"/>
+      <c r="H762" s="15" t="n"/>
+      <c r="I762" s="15" t="n"/>
+      <c r="J762" s="15" t="n"/>
+      <c r="K762" s="15" t="n"/>
+      <c r="L762" s="22" t="n"/>
+      <c r="M762" s="22" t="n"/>
+      <c r="N762" s="22" t="n"/>
+      <c r="O762" s="22" t="n"/>
+      <c r="P762" s="22" t="n"/>
+      <c r="Q762" s="22" t="n"/>
+      <c r="R762" s="22" t="n"/>
     </row>
     <row r="763" hidden="1" ht="135" customHeight="1">
-      <c r="A763" s="10" t="inlineStr">
-        <is>
-          <t>MAC</t>
-        </is>
-      </c>
-      <c r="B763" s="8" t="inlineStr">
-        <is>
-          <t>0003</t>
-        </is>
-      </c>
-      <c r="C763" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D763" s="12" t="n">
-        <v>400</v>
-      </c>
-      <c r="E763" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="F763" s="29" t="inlineStr">
-        <is>
-          <t>mm/s</t>
-        </is>
-      </c>
-      <c r="G763" s="29" t="n"/>
-      <c r="H763" s="29" t="inlineStr">
-        <is>
-          <t>R/W</t>
-        </is>
-      </c>
-      <c r="I763" s="29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J763" s="29" t="inlineStr">
-        <is>
-          <t>uint16</t>
-        </is>
-      </c>
-      <c r="K763" s="29" t="inlineStr">
-        <is>
-          <t>Temporaere Vorzugsgeschwindigkeit</t>
-        </is>
-      </c>
-      <c r="L763" s="28" t="n"/>
-      <c r="M763" s="28" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N763" s="28" t="inlineStr">
-        <is>
-          <t>Sollgeschwindigkeit fuer kontinuierlichen und getakteten IBN-Testbetrieb</t>
-        </is>
-      </c>
-      <c r="O763" s="28" t="n"/>
-      <c r="P763" s="28" t="n"/>
-      <c r="Q763" s="28" t="n"/>
-      <c r="R763" s="28" t="inlineStr">
-        <is>
-          <t>KI: Ich verstehe MAC0003 als temporaere Vorzugsgeschwindigkeit fuer Motor 3 im IBN-Test. Wird kein neuer Wert gesetzt, verwendet der Raspi den zuletzt gespeicherten Wert. Produktiv wird die Geschwindigkeit ueber MAP0014 bzw. die Betriebsart vorgegeben. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-      <c r="S763" s="4" t="n"/>
-      <c r="T763" s="4" t="n"/>
-      <c r="U763" s="4" t="n"/>
+      <c r="A763" s="10" t="n"/>
+      <c r="B763" s="8" t="n"/>
+      <c r="C763" s="43" t="n"/>
+      <c r="D763" s="11" t="n"/>
+      <c r="E763" s="11" t="n"/>
+      <c r="F763" s="15" t="n"/>
+      <c r="G763" s="15" t="n"/>
+      <c r="H763" s="15" t="n"/>
+      <c r="I763" s="15" t="n"/>
+      <c r="J763" s="15" t="n"/>
+      <c r="K763" s="15" t="n"/>
+      <c r="L763" s="22" t="n"/>
+      <c r="M763" s="22" t="n"/>
+      <c r="N763" s="22" t="n"/>
+      <c r="O763" s="22" t="n"/>
+      <c r="P763" s="22" t="n"/>
+      <c r="Q763" s="22" t="n"/>
+      <c r="R763" s="22" t="n"/>
     </row>
     <row r="764" hidden="1" ht="135" customHeight="1">
-      <c r="A764" s="10" t="inlineStr">
-        <is>
-          <t>MAC</t>
-        </is>
-      </c>
-      <c r="B764" s="8" t="inlineStr">
-        <is>
-          <t>0004</t>
-        </is>
-      </c>
-      <c r="C764" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D764" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E764" s="12" t="n">
-        <v>300</v>
-      </c>
-      <c r="F764" s="29" t="inlineStr">
-        <is>
-          <t>mm/s2</t>
-        </is>
-      </c>
-      <c r="G764" s="29" t="n"/>
-      <c r="H764" s="29" t="inlineStr">
-        <is>
-          <t>R/W</t>
-        </is>
-      </c>
-      <c r="I764" s="29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J764" s="29" t="inlineStr">
-        <is>
-          <t>uint16</t>
-        </is>
-      </c>
-      <c r="K764" s="29" t="inlineStr">
-        <is>
-          <t>Temporaere Transport-Rampe</t>
-        </is>
-      </c>
-      <c r="L764" s="28" t="n"/>
-      <c r="M764" s="28" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N764" s="28" t="inlineStr">
-        <is>
-          <t>Beschleunigung/Verzoegerung fuer Motor 3 im IBN-Testbetrieb</t>
-        </is>
-      </c>
-      <c r="O764" s="28" t="n"/>
-      <c r="P764" s="28" t="n"/>
-      <c r="Q764" s="28" t="n"/>
-      <c r="R764" s="28" t="inlineStr">
-        <is>
-          <t>KI: Ich verstehe MAC0004 als temporaere Rampe fuer Beschleunigung und Bremsung des Etikettenantriebs im IBN-Test. Produktiv wird diese Vorgabe aus Maschinen- bzw. Formatparametern abgeleitet und darf den Etikettenschlupf nicht erhoehen. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: mm/s2. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-      <c r="S764" s="4" t="n"/>
-      <c r="T764" s="4" t="n"/>
-      <c r="U764" s="4" t="n"/>
+      <c r="A764" s="10" t="n"/>
+      <c r="B764" s="8" t="n"/>
+      <c r="C764" s="43" t="n"/>
+      <c r="D764" s="11" t="n"/>
+      <c r="E764" s="11" t="n"/>
+      <c r="F764" s="15" t="n"/>
+      <c r="G764" s="15" t="n"/>
+      <c r="H764" s="15" t="n"/>
+      <c r="I764" s="15" t="n"/>
+      <c r="J764" s="15" t="n"/>
+      <c r="K764" s="15" t="n"/>
+      <c r="L764" s="22" t="n"/>
+      <c r="M764" s="22" t="n"/>
+      <c r="N764" s="22" t="n"/>
+      <c r="O764" s="22" t="n"/>
+      <c r="P764" s="22" t="n"/>
+      <c r="Q764" s="22" t="n"/>
+      <c r="R764" s="22" t="n"/>
     </row>
     <row r="765" hidden="1" ht="135" customHeight="1">
-      <c r="A765" s="10" t="inlineStr">
-        <is>
-          <t>MAC</t>
-        </is>
-      </c>
-      <c r="B765" s="8" t="inlineStr">
-        <is>
-          <t>0005</t>
-        </is>
-      </c>
-      <c r="C765" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="D765" s="12" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E765" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F765" s="29" t="inlineStr">
-        <is>
-          <t>1/10mm</t>
-        </is>
-      </c>
-      <c r="G765" s="29" t="n"/>
-      <c r="H765" s="29" t="inlineStr">
-        <is>
-          <t>R/W</t>
-        </is>
-      </c>
-      <c r="I765" s="29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J765" s="29" t="inlineStr">
-        <is>
-          <t>uint32</t>
-        </is>
-      </c>
-      <c r="K765" s="29" t="inlineStr">
-        <is>
-          <t>Temporaere kontinuierliche Weglaenge</t>
-        </is>
-      </c>
-      <c r="L765" s="28" t="n"/>
-      <c r="M765" s="28" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N765" s="28" t="inlineStr">
-        <is>
-          <t>Weg fuer kontinuierliches Vorziehen/Rueckspulen; 0=endlos bis Stop</t>
-        </is>
-      </c>
-      <c r="O765" s="28" t="n"/>
-      <c r="P765" s="28" t="n"/>
-      <c r="Q765" s="28" t="n"/>
-      <c r="R765" s="28" t="inlineStr">
-        <is>
-          <t>KI: Ich verstehe MAC0005 als temporaere Wegvorgabe fuer kontinuierliches Vorziehen oder Rueckspulen. Default 0 bedeutet endlos fahren bis MAC0001=0. Produktiv wird diese Laenge aus Ablaufzustand, Rueckspulweg oder Bedienhandlung bestimmt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: 1/10mm. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-      <c r="S765" s="4" t="n"/>
-      <c r="T765" s="4" t="n"/>
-      <c r="U765" s="4" t="n"/>
+      <c r="A765" s="10" t="n"/>
+      <c r="B765" s="8" t="n"/>
+      <c r="C765" s="43" t="n"/>
+      <c r="D765" s="11" t="n"/>
+      <c r="E765" s="11" t="n"/>
+      <c r="F765" s="15" t="n"/>
+      <c r="G765" s="15" t="n"/>
+      <c r="H765" s="15" t="n"/>
+      <c r="I765" s="15" t="n"/>
+      <c r="J765" s="15" t="n"/>
+      <c r="K765" s="15" t="n"/>
+      <c r="L765" s="22" t="n"/>
+      <c r="M765" s="22" t="n"/>
+      <c r="N765" s="22" t="n"/>
+      <c r="O765" s="22" t="n"/>
+      <c r="P765" s="22" t="n"/>
+      <c r="Q765" s="22" t="n"/>
+      <c r="R765" s="22" t="n"/>
     </row>
     <row r="766" hidden="1">
-      <c r="A766" s="10" t="inlineStr">
-        <is>
-          <t>MAC</t>
-        </is>
-      </c>
-      <c r="B766" s="8" t="inlineStr">
-        <is>
-          <t>0006</t>
-        </is>
-      </c>
-      <c r="C766" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="D766" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E766" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="F766" s="29" t="inlineStr">
-        <is>
-          <t>Zyklen</t>
-        </is>
-      </c>
-      <c r="G766" s="29" t="n"/>
-      <c r="H766" s="29" t="inlineStr">
-        <is>
-          <t>R/W</t>
-        </is>
-      </c>
-      <c r="I766" s="29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J766" s="29" t="inlineStr">
-        <is>
-          <t>uint16</t>
-        </is>
-      </c>
-      <c r="K766" s="29" t="inlineStr">
-        <is>
-          <t>Temporaere Taktzyklus-Anzahl</t>
-        </is>
-      </c>
-      <c r="L766" s="28" t="n"/>
-      <c r="M766" s="28" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="N766" s="28" t="inlineStr">
-        <is>
-          <t>Anzahl Takte im Testbetrieb; 0=endlos bis Stop</t>
-        </is>
-      </c>
-      <c r="O766" s="28" t="n"/>
-      <c r="P766" s="28" t="n"/>
-      <c r="Q766" s="28" t="n"/>
-      <c r="R766" s="28" t="inlineStr">
-        <is>
-          <t>KI: Ich verstehe MAC0006 als temporaere Zyklusanzahl fuer den getakteten IBN-Test. Default 20 entspricht einem kurzen Stabilitaetstest; 0 bedeutet laufender Taktbetrieb bis MAC0001=0. Spaeter wird diese Logik durch den echten Produktionsablauf und das Schieberegister ersetzt. Microtom soll diesen Wert lesen und bei Bedarf auch schreiben koennen. Der ESP soll ihn gemaess Masterliste nicht verwenden. Einheit bzw. Wertebereich laut Tabelle: Zyklen. Der Wert ist laut Tabelle nicht formatrelevant und eher als Maschinen-/Systemeinstellung zu sehen.</t>
-        </is>
-      </c>
-      <c r="S766" s="4" t="n"/>
-      <c r="T766" s="4" t="n"/>
-      <c r="U766" s="4" t="n"/>
+      <c r="A766" s="10" t="n"/>
+      <c r="B766" s="8" t="n"/>
+      <c r="C766" s="43" t="n"/>
+      <c r="D766" s="11" t="n"/>
+      <c r="E766" s="11" t="n"/>
+      <c r="F766" s="15" t="n"/>
+      <c r="G766" s="15" t="n"/>
+      <c r="H766" s="15" t="n"/>
+      <c r="I766" s="15" t="n"/>
+      <c r="J766" s="15" t="n"/>
+      <c r="K766" s="15" t="n"/>
+      <c r="L766" s="22" t="n"/>
+      <c r="M766" s="22" t="n"/>
+      <c r="N766" s="22" t="n"/>
+      <c r="O766" s="22" t="n"/>
+      <c r="P766" s="22" t="n"/>
+      <c r="Q766" s="22" t="n"/>
+      <c r="R766" s="22" t="n"/>
     </row>
     <row r="767" hidden="1">
       <c r="A767" s="10" t="n"/>
@@ -58595,126 +58305,9 @@
       <c r="Q775" s="22" t="n"/>
       <c r="R775" s="22" t="n"/>
     </row>
-    <row r="776" hidden="1">
-      <c r="A776" s="10" t="n"/>
-      <c r="B776" s="8" t="n"/>
-      <c r="C776" s="43" t="n"/>
-      <c r="D776" s="11" t="n"/>
-      <c r="E776" s="11" t="n"/>
-      <c r="F776" s="15" t="n"/>
-      <c r="G776" s="15" t="n"/>
-      <c r="H776" s="15" t="n"/>
-      <c r="I776" s="15" t="n"/>
-      <c r="J776" s="15" t="n"/>
-      <c r="K776" s="15" t="n"/>
-      <c r="L776" s="22" t="n"/>
-      <c r="M776" s="22" t="n"/>
-      <c r="N776" s="22" t="n"/>
-      <c r="O776" s="22" t="n"/>
-      <c r="P776" s="22" t="n"/>
-      <c r="Q776" s="22" t="n"/>
-      <c r="R776" s="22" t="n"/>
-    </row>
-    <row r="777" hidden="1">
-      <c r="A777" s="10" t="n"/>
-      <c r="B777" s="8" t="n"/>
-      <c r="C777" s="43" t="n"/>
-      <c r="D777" s="11" t="n"/>
-      <c r="E777" s="11" t="n"/>
-      <c r="F777" s="15" t="n"/>
-      <c r="G777" s="15" t="n"/>
-      <c r="H777" s="15" t="n"/>
-      <c r="I777" s="15" t="n"/>
-      <c r="J777" s="15" t="n"/>
-      <c r="K777" s="15" t="n"/>
-      <c r="L777" s="22" t="n"/>
-      <c r="M777" s="22" t="n"/>
-      <c r="N777" s="22" t="n"/>
-      <c r="O777" s="22" t="n"/>
-      <c r="P777" s="22" t="n"/>
-      <c r="Q777" s="22" t="n"/>
-      <c r="R777" s="22" t="n"/>
-    </row>
-    <row r="778" hidden="1">
-      <c r="A778" s="10" t="n"/>
-      <c r="B778" s="8" t="n"/>
-      <c r="C778" s="43" t="n"/>
-      <c r="D778" s="11" t="n"/>
-      <c r="E778" s="11" t="n"/>
-      <c r="F778" s="15" t="n"/>
-      <c r="G778" s="15" t="n"/>
-      <c r="H778" s="15" t="n"/>
-      <c r="I778" s="15" t="n"/>
-      <c r="J778" s="15" t="n"/>
-      <c r="K778" s="15" t="n"/>
-      <c r="L778" s="22" t="n"/>
-      <c r="M778" s="22" t="n"/>
-      <c r="N778" s="22" t="n"/>
-      <c r="O778" s="22" t="n"/>
-      <c r="P778" s="22" t="n"/>
-      <c r="Q778" s="22" t="n"/>
-      <c r="R778" s="22" t="n"/>
-    </row>
-    <row r="779">
-      <c r="A779" s="10" t="n"/>
-      <c r="B779" s="8" t="n"/>
-      <c r="C779" s="43" t="n"/>
-      <c r="D779" s="11" t="n"/>
-      <c r="E779" s="11" t="n"/>
-      <c r="F779" s="15" t="n"/>
-      <c r="G779" s="15" t="n"/>
-      <c r="H779" s="15" t="n"/>
-      <c r="I779" s="15" t="n"/>
-      <c r="J779" s="15" t="n"/>
-      <c r="K779" s="15" t="n"/>
-      <c r="L779" s="22" t="n"/>
-      <c r="M779" s="22" t="n"/>
-      <c r="N779" s="22" t="n"/>
-      <c r="O779" s="22" t="n"/>
-      <c r="P779" s="22" t="n"/>
-      <c r="Q779" s="22" t="n"/>
-      <c r="R779" s="22" t="n"/>
-    </row>
-    <row r="780">
-      <c r="A780" s="10" t="n"/>
-      <c r="B780" s="8" t="n"/>
-      <c r="C780" s="43" t="n"/>
-      <c r="D780" s="11" t="n"/>
-      <c r="E780" s="11" t="n"/>
-      <c r="F780" s="15" t="n"/>
-      <c r="G780" s="15" t="n"/>
-      <c r="H780" s="15" t="n"/>
-      <c r="I780" s="15" t="n"/>
-      <c r="J780" s="15" t="n"/>
-      <c r="K780" s="15" t="n"/>
-      <c r="L780" s="22" t="n"/>
-      <c r="M780" s="22" t="n"/>
-      <c r="N780" s="22" t="n"/>
-      <c r="O780" s="22" t="n"/>
-      <c r="P780" s="22" t="n"/>
-      <c r="Q780" s="22" t="n"/>
-      <c r="R780" s="22" t="n"/>
-    </row>
-    <row r="781">
-      <c r="A781" s="10" t="n"/>
-      <c r="B781" s="8" t="n"/>
-      <c r="C781" s="43" t="n"/>
-      <c r="D781" s="11" t="n"/>
-      <c r="E781" s="11" t="n"/>
-      <c r="F781" s="15" t="n"/>
-      <c r="G781" s="15" t="n"/>
-      <c r="H781" s="15" t="n"/>
-      <c r="I781" s="15" t="n"/>
-      <c r="J781" s="15" t="n"/>
-      <c r="K781" s="15" t="n"/>
-      <c r="L781" s="22" t="n"/>
-      <c r="M781" s="22" t="n"/>
-      <c r="N781" s="22" t="n"/>
-      <c r="O781" s="22" t="n"/>
-      <c r="P781" s="22" t="n"/>
-      <c r="Q781" s="22" t="n"/>
-      <c r="R781" s="22" t="n"/>
-    </row>
+    <row r="776" hidden="1"/>
+    <row r="777" hidden="1"/>
+    <row r="778" hidden="1"/>
   </sheetData>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation sqref="M1:M1048576 P2:P119" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -58730,4 +58323,296 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a32518fee107c04aa9bd7948c0d3f18">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e97db55af52189d57b3fce0d0bdbaea8" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
+    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFC6A37-2F19-49DF-87E6-AB5652B8C8E4}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC4971B4-DAD3-46DF-A3E3-9AF4554EE247}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B6A060-7507-475D-9722-2354344567E1}"/>
 </file>
</xml_diff>

<commit_message>
Make motor setup values authoritative
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -51101,10 +51101,10 @@
         <v>0</v>
       </c>
       <c r="D664" s="11" t="n">
-        <v>2100</v>
+        <v>1540</v>
       </c>
       <c r="E664" s="11" t="n">
-        <v>1550</v>
+        <v>1535</v>
       </c>
       <c r="F664" s="15" t="inlineStr">
         <is>
@@ -51164,13 +51164,13 @@
         </is>
       </c>
       <c r="C665" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="D665" s="11" t="n">
-        <v>10000</v>
+        <v>990</v>
       </c>
       <c r="E665" s="11" t="n">
-        <v>980</v>
+        <v>990</v>
       </c>
       <c r="F665" s="15" t="inlineStr">
         <is>
@@ -51438,7 +51438,7 @@
         <v>650</v>
       </c>
       <c r="E669" s="11" t="n">
-        <v>300</v>
+        <v>-200</v>
       </c>
       <c r="F669" s="15" t="inlineStr">
         <is>
@@ -51504,7 +51504,7 @@
         <v>650</v>
       </c>
       <c r="E670" s="11" t="n">
-        <v>300</v>
+        <v>-200</v>
       </c>
       <c r="F670" s="15" t="inlineStr">
         <is>
@@ -51567,10 +51567,10 @@
         <v>100</v>
       </c>
       <c r="D671" s="11" t="n">
-        <v>910</v>
+        <v>1000</v>
       </c>
       <c r="E671" s="11" t="n">
-        <v>910</v>
+        <v>925</v>
       </c>
       <c r="F671" s="15" t="inlineStr">
         <is>
@@ -51633,7 +51633,7 @@
         <v>100</v>
       </c>
       <c r="D672" s="11" t="n">
-        <v>910</v>
+        <v>1000</v>
       </c>
       <c r="E672" s="11" t="n">
         <v>910</v>
@@ -52581,10 +52581,10 @@
         <v>0</v>
       </c>
       <c r="D686" s="11" t="n">
-        <v>2100</v>
+        <v>1540</v>
       </c>
       <c r="E686" s="11" t="n">
-        <v>1550</v>
+        <v>1535</v>
       </c>
       <c r="F686" s="15" t="inlineStr">
         <is>
@@ -52644,13 +52644,13 @@
         </is>
       </c>
       <c r="C687" s="3" t="n">
-        <v>-10000</v>
+        <v>0</v>
       </c>
       <c r="D687" s="11" t="n">
-        <v>10000</v>
+        <v>990</v>
       </c>
       <c r="E687" s="11" t="n">
-        <v>980</v>
+        <v>990</v>
       </c>
       <c r="F687" s="15" t="inlineStr">
         <is>
@@ -52716,7 +52716,7 @@
         <v>650</v>
       </c>
       <c r="E688" s="11" t="n">
-        <v>300</v>
+        <v>-200</v>
       </c>
       <c r="F688" s="15" t="inlineStr">
         <is>
@@ -52782,7 +52782,7 @@
         <v>650</v>
       </c>
       <c r="E689" s="11" t="n">
-        <v>300</v>
+        <v>-200</v>
       </c>
       <c r="F689" s="15" t="inlineStr">
         <is>
@@ -52845,7 +52845,7 @@
         <v>100</v>
       </c>
       <c r="D690" s="11" t="n">
-        <v>910</v>
+        <v>1000</v>
       </c>
       <c r="E690" s="11" t="n">
         <v>910</v>
@@ -52911,10 +52911,10 @@
         <v>100</v>
       </c>
       <c r="D691" s="11" t="n">
-        <v>910</v>
+        <v>1000</v>
       </c>
       <c r="E691" s="11" t="n">
-        <v>910</v>
+        <v>925</v>
       </c>
       <c r="F691" s="15" t="inlineStr">
         <is>
@@ -58606,13 +58606,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFC6A37-2F19-49DF-87E6-AB5652B8C8E4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{581018F7-B077-41F8-932C-95F125681D77}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC4971B4-DAD3-46DF-A3E3-9AF4554EE247}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75BA8AE4-C304-4D21-904A-1D0430EAC1A5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82B6A060-7507-475D-9722-2354344567E1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A4D9519-4D37-46AB-809E-0405F788D2A2}"/>
 </file>
</xml_diff>

<commit_message>
Handle production pause without purge fault
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -51173,7 +51173,7 @@
       </c>
       <c r="E665" s="11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F665" s="15" t="inlineStr">
@@ -51447,7 +51447,7 @@
       </c>
       <c r="E669" s="11" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>598</t>
         </is>
       </c>
       <c r="F669" s="15" t="inlineStr">
@@ -53320,7 +53320,7 @@
       </c>
       <c r="E696" s="11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F696" s="15" t="inlineStr">
@@ -53388,7 +53388,7 @@
       </c>
       <c r="E697" s="11" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>598</t>
         </is>
       </c>
       <c r="F697" s="15" t="inlineStr">
@@ -59292,13 +59292,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFF60DE0-9F1E-42B1-B544-2CDA6286C584}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3004EFEF-C355-4181-B29E-DA5E0E831C7D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A3F50B1-B11B-43FB-97A4-F70B5A5AC586}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D25AFB-E4B2-4A92-910D-8F020805505A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5C0D531-FD48-4D9B-9E4E-6AFFEFD41BA8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{473561A7-989C-4EE1-959B-8A7E6E682277}"/>
 </file>
</xml_diff>

<commit_message>
Make production marker distances editable
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -48441,7 +48441,7 @@
       </c>
       <c r="E627" s="6" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>5970</t>
         </is>
       </c>
       <c r="F627" s="15" t="inlineStr">
@@ -59003,302 +59003,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
-    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
-    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3004EFEF-C355-4181-B29E-DA5E0E831C7D}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D25AFB-E4B2-4A92-910D-8F020805505A}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{473561A7-989C-4EE1-959B-8A7E6E682277}"/>
 </file>
</xml_diff>

<commit_message>
Sync parameter master from running Raspi
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -48441,7 +48441,7 @@
       </c>
       <c r="E627" s="6" t="inlineStr">
         <is>
-          <t>5970</t>
+          <t>6010</t>
         </is>
       </c>
       <c r="F627" s="15" t="inlineStr">
@@ -48513,7 +48513,7 @@
       </c>
       <c r="E628" s="7" t="inlineStr">
         <is>
-          <t>8500</t>
+          <t>7800</t>
         </is>
       </c>
       <c r="F628" s="31" t="inlineStr">
@@ -51105,7 +51105,7 @@
       </c>
       <c r="E664" s="11" t="inlineStr">
         <is>
-          <t>1540</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F664" s="15" t="inlineStr">
@@ -51818,8 +51818,10 @@
       <c r="D675" s="12" t="n">
         <v>15000</v>
       </c>
-      <c r="E675" s="12" t="n">
-        <v>9600</v>
+      <c r="E675" s="12" t="inlineStr">
+        <is>
+          <t>9600</t>
+        </is>
       </c>
       <c r="F675" s="29" t="inlineStr">
         <is>
@@ -53252,7 +53254,7 @@
       </c>
       <c r="E695" s="11" t="inlineStr">
         <is>
-          <t>1540</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F695" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Stabilize ESP command communication
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -59005,4 +59005,302 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
+    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8890953C-96EE-40CF-BA4A-BFEBBC839B03}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{461F2087-9DDD-46D2-833B-A8BDD8425AD0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77185E60-849B-46ED-A06B-2C03FBCFB2B7}"/>
 </file>
</xml_diff>

<commit_message>
Handle Wickler fill thresholds and continuous resume
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -48873,7 +48873,7 @@
       </c>
       <c r="E633" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F633" s="15" t="inlineStr">
@@ -59005,302 +59005,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
-    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
-    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8890953C-96EE-40CF-BA4A-BFEBBC839B03}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{461F2087-9DDD-46D2-833B-A8BDD8425AD0}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77185E60-849B-46ED-A06B-2C03FBCFB2B7}"/>
 </file>
</xml_diff>

<commit_message>
Sync master workbook with TTO format
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="rng_Lieferanten">#REF!</definedName>
@@ -41673,7 +41673,7 @@
       </c>
       <c r="E531" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F531" s="15" t="inlineStr">
@@ -42669,7 +42669,7 @@
       </c>
       <c r="E545" s="11" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F545" s="15" t="inlineStr">
@@ -42745,7 +42745,7 @@
       </c>
       <c r="E546" s="11" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F546" s="15" t="inlineStr">
@@ -42893,7 +42893,7 @@
       </c>
       <c r="E548" s="11" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>151</t>
         </is>
       </c>
       <c r="F548" s="15" t="inlineStr">
@@ -47113,7 +47113,7 @@
       </c>
       <c r="E609" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>380</t>
         </is>
       </c>
       <c r="F609" s="15" t="inlineStr">
@@ -47185,7 +47185,7 @@
       </c>
       <c r="E610" s="7" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1045</t>
         </is>
       </c>
       <c r="F610" s="31" t="inlineStr">
@@ -47553,7 +47553,7 @@
       </c>
       <c r="E615" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F615" s="15" t="inlineStr">
@@ -47625,7 +47625,7 @@
       </c>
       <c r="E616" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F616" s="31" t="inlineStr">
@@ -47697,7 +47697,7 @@
       </c>
       <c r="E617" s="6" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F617" s="15" t="inlineStr">
@@ -47769,7 +47769,7 @@
       </c>
       <c r="E618" s="7" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F618" s="31" t="inlineStr">
@@ -47845,7 +47845,7 @@
       </c>
       <c r="E619" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90.55</t>
         </is>
       </c>
       <c r="F619" s="15" t="inlineStr">
@@ -48149,7 +48149,7 @@
       </c>
       <c r="E623" s="6" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F623" s="15" t="inlineStr">
@@ -49957,7 +49957,7 @@
       </c>
       <c r="E648" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F648" s="15" t="inlineStr">
@@ -59005,4 +59005,302 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
+    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA816280-568C-49A5-B581-050D82F75246}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{414F502C-C4B5-4113-86CA-7EBA872E50D0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F846312-43FB-4542-891C-994562E22FAB}"/>
 </file>
</xml_diff>

<commit_message>
Sync live Databridge production workbook
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Parameter" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="rng_Lieferanten">#REF!</definedName>
@@ -48297,7 +48297,7 @@
       </c>
       <c r="E625" s="6" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>910</t>
         </is>
       </c>
       <c r="F625" s="15" t="inlineStr">
@@ -59005,302 +59005,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
-    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
-    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA816280-568C-49A5-B581-050D82F75246}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{414F502C-C4B5-4113-86CA-7EBA872E50D0}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F846312-43FB-4542-891C-994562E22FAB}"/>
 </file>
</xml_diff>

<commit_message>
Use MAP0014 for setup transport speed
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -48073,7 +48073,7 @@
       </c>
       <c r="E622" s="7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F622" s="31" t="inlineStr">
@@ -59005,4 +59005,302 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
+    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0A3B0F1-1E4E-4508-8BE4-9BF4693761CF}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB4959D0-53E8-49D4-A3E3-F6734294744A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93F46591-B842-4412-8E3F-2B5549EFED20}"/>
 </file>
</xml_diff>

<commit_message>
Align live Databridge state
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -48441,7 +48441,7 @@
       </c>
       <c r="E627" s="6" t="inlineStr">
         <is>
-          <t>6010</t>
+          <t>6910</t>
         </is>
       </c>
       <c r="F627" s="15" t="inlineStr">
@@ -59005,302 +59005,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="af0d30918d172d53a6c97a3e981f1432">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c8b33fdf811bb6ef4bbd77ea5570dd7f" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
-    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
-    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0A3B0F1-1E4E-4508-8BE4-9BF4693761CF}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB4959D0-53E8-49D4-A3E3-F6734294744A}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93F46591-B842-4412-8E3F-2B5549EFED20}"/>
 </file>
</xml_diff>

<commit_message>
Stabilize ESP communication and setup wickler hints
</commit_message>
<xml_diff>
--- a/master_data/Parameterliste SAR41-MAS-004.xlsx
+++ b/master_data/Parameterliste SAR41-MAS-004.xlsx
@@ -51214,10 +51214,8 @@
           <t>0057</t>
         </is>
       </c>
-      <c r="C665" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C665" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D665" s="11" t="n">
         <v>990</v>
@@ -53825,10 +53823,8 @@
           <t>0012</t>
         </is>
       </c>
-      <c r="C702" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="C702" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D702" s="11" t="n">
         <v>990</v>

</xml_diff>